<commit_message>
[mp006] docs: refresh owner xlsx+docx with 2026-05-10 status
- Add 3 new owner-visible items: cross-route data parity check,
  product-line dashboard view (34-col Excel lift), shipping label
  status with reference photos
- Refresh narrative with staging-operational + first end-to-end
  green milestone (12/12 demo orders complete roundtrip)
- Extend xlsx schema with column J "JIRA" for upcoming back-linked
  issue keys (loaded from sidecar jira_keys.json)
- Catalog count: 97 -> 100 work items
</commit_message>
<xml_diff>
--- a/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
+++ b/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hang_Muc_Cong_Viec" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hang_Muc_Cong_Viec'!$A$1:$I$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Hang_Muc_Cong_Viec'!$A$1:$J$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -821,7 +821,7 @@
         </is>
       </c>
       <c r="C28" s="7">
-        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H98,"Chưa bắt đầu")</f>
+        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H101,"Chưa bắt đầu")</f>
         <v/>
       </c>
     </row>
@@ -832,7 +832,7 @@
         </is>
       </c>
       <c r="C29" s="7">
-        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H98,"Đang làm")</f>
+        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H101,"Đang làm")</f>
         <v/>
       </c>
     </row>
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C30" s="7">
-        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H98,"Hoàn thành")</f>
+        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H101,"Hoàn thành")</f>
         <v/>
       </c>
     </row>
@@ -854,7 +854,7 @@
         </is>
       </c>
       <c r="C31" s="7">
-        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H98,"Chặn")</f>
+        <f>COUNTIF(Hang_Muc_Cong_Viec!H2:H101,"Chặn")</f>
         <v/>
       </c>
     </row>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="C32" s="9">
-        <f>COUNTA(Hang_Muc_Cong_Viec!C2:C98)</f>
+        <f>COUNTA(Hang_Muc_Cong_Viec!C2:C101)</f>
         <v/>
       </c>
     </row>
@@ -889,7 +889,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I98"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -901,6 +901,7 @@
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="35" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -949,6 +950,11 @@
           <t>Ghi chú</t>
         </is>
       </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>JIRA</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="7" t="n">
@@ -990,6 +996,7 @@
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr"/>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="7" t="n">
@@ -1031,6 +1038,7 @@
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="7" t="n">
@@ -1072,6 +1080,7 @@
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
+      <c r="J4" s="7" t="inlineStr"/>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="7" t="n">
@@ -1113,6 +1122,7 @@
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="7" t="n">
@@ -1154,6 +1164,7 @@
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="7" t="n">
@@ -1195,6 +1206,7 @@
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -1236,6 +1248,7 @@
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -1277,6 +1290,7 @@
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -1289,27 +1303,27 @@
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Xuất Excel tin nhắn khách theo khoảng thời gian</t>
+          <t>Đối chiếu dữ liệu giữa đường chính và đường dự phòng</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Marketing chọn khoảng thời gian, bấm 'Xuất tin nhắn' để tải Excel tất cả tin nhắn khách.</t>
+          <t>Sau mỗi đợt đồng bộ, hệ thống so sánh đơn lấy từ kết nối Etsy chính thức với đơn lấy từ email dự phòng để bảo đảm 100% trùng khớp về số đơn, sản phẩm, giá, người nhận và phí vận chuyển. Sai lệch được liệt kê trên một trang riêng cho BA xử lý.</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
@@ -1317,7 +1331,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Đã đối chiếu thành công 12/12 đơn mẫu trên môi trường demo.</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -1325,32 +1344,32 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>2. Làm sạch dữ liệu đơn hàng cũ</t>
+          <t>1. Đồng bộ đơn hàng từ Etsy</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Nhập 17.659 đơn hàng cũ từ file Excel</t>
+          <t>Xuất Excel tin nhắn khách theo khoảng thời gian</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Admin tải file Excel lịch sử lên; hệ thống đọc và tạo đơn. Có thể tiếp tục từ điểm dừng nếu bị gián đoạn.</t>
+          <t>Marketing chọn khoảng thời gian, bấm 'Xuất tin nhắn' để tải Excel tất cả tin nhắn khách.</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
@@ -1359,6 +1378,7 @@
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -1371,17 +1391,17 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Sửa 423 đơn ghi giá 0 USD</t>
+          <t>Nhập 17.659 đơn hàng cũ từ file Excel</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống tự tính lại giá từ nguồn; đơn không khôi phục được sẽ liệt kê cho BA xử lý tay.</t>
+          <t>Admin tải file Excel lịch sử lên; hệ thống đọc và tạo đơn. Có thể tiếp tục từ điểm dừng nếu bị gián đoạn.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Kiểm soát giá</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -1400,6 +1420,7 @@
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
+      <c r="J12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -1412,12 +1433,12 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Nhận đúng tiền tệ USD/EUR/GBP/CAD/VND</t>
+          <t>Sửa 423 đơn ghi giá 0 USD</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Đọc ký hiệu tiền tệ ($, €, £, C$, ₫) và gán đúng cho từng đơn. Đơn vẫn giữ tiền gốc.</t>
+          <t>Hệ thống tự tính lại giá từ nguồn; đơn không khôi phục được sẽ liệt kê cho BA xử lý tay.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1441,6 +1462,7 @@
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="7" t="n">
@@ -1453,12 +1475,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Tách phí ship thành dòng riêng</t>
+          <t>Nhận đúng tiền tệ USD/EUR/GBP/CAD/VND</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Mỗi đơn có dòng 'Phí vận chuyển Etsy' riêng để tổng đơn khớp nguồn trong sai số 0,01 USD.</t>
+          <t>Đọc ký hiệu tiền tệ ($, €, £, C$, ₫) và gán đúng cho từng đơn. Đơn vẫn giữ tiền gốc.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1482,6 +1504,7 @@
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
+      <c r="J14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="7" t="n">
@@ -1494,17 +1517,17 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Gộp khách hàng trùng có BA duyệt</t>
+          <t>Tách phí ship thành dòng riêng</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống đề xuất danh sách khách hàng nghi trùng, xuất Excel, BA tích chọn rồi tải lên để gộp. Hệ thống KHÔNG tự gộp.</t>
+          <t>Mỗi đơn có dòng 'Phí vận chuyển Etsy' riêng để tổng đơn khớp nguồn trong sai số 0,01 USD.</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Kiểm soát giá</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1523,6 +1546,7 @@
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="7" t="n">
@@ -1535,17 +1559,17 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>Báo cáo đối chiếu sau khi làm sạch dữ liệu</t>
+          <t>Gộp khách hàng trùng có BA duyệt</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Sau khi chạy xong, hệ thống xuất báo cáo: tổng đơn, doanh thu, phí ship, đơn lỗi. BA Lead ký xác nhận trước khi sang giai đoạn tiếp theo.</t>
+          <t>Hệ thống đề xuất danh sách khách hàng nghi trùng, xuất Excel, BA tích chọn rồi tải lên để gộp. Hệ thống KHÔNG tự gộp.</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án, BA</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -1564,6 +1588,7 @@
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="7" t="n">
@@ -1576,17 +1601,17 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Đặt đơn cũ ở trạng thái 'đã hoàn tất'</t>
+          <t>Báo cáo đối chiếu sau khi làm sạch dữ liệu</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Toàn bộ 17.659 đơn cũ được mặc định trạng thái 'đã hoàn tất' và để ngoài pipeline sản xuất hiện tại; admin có thể chuyển vào pipeline 'Lưu trữ' nếu muốn.</t>
+          <t>Sau khi chạy xong, hệ thống xuất báo cáo: tổng đơn, doanh thu, phí ship, đơn lỗi. BA Lead ký xác nhận trước khi sang giai đoạn tiếp theo.</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>Chủ dự án, BA</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -1605,6 +1630,7 @@
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="7" t="n">
@@ -1612,22 +1638,22 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>3. Bảng điều khiển Đơn hàng</t>
+          <t>2. Làm sạch dữ liệu đơn hàng cũ</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Hiển thị 10 cột chính</t>
+          <t>Đặt đơn cũ ở trạng thái 'đã hoàn tất'</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Cửa hàng, Mã đơn, Tracking, Ảnh, Ngày, Tình trạng, Số lượng, Dịch vụ vận chuyển, Quốc gia, Tổng tiền.</t>
+          <t>Toàn bộ 17.659 đơn cũ được mặc định trạng thái 'đã hoàn tất' và để ngoài pipeline sản xuất hiện tại; admin có thể chuyển vào pipeline 'Lưu trữ' nếu muốn.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
@@ -1646,6 +1672,7 @@
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
+      <c r="J18" s="7" t="inlineStr"/>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="7" t="n">
@@ -1658,12 +1685,12 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Cửa hàng và Mã đơn ở 2 cột đầu, có ô tìm kiếm</t>
+          <t>Hiển thị 10 cột chính</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Search hoạt động trên cả Cửa hàng và Mã đơn.</t>
+          <t>Cửa hàng, Mã đơn, Tracking, Ảnh, Ngày, Tình trạng, Số lượng, Dịch vụ vận chuyển, Quốc gia, Tổng tiền.</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -1673,7 +1700,7 @@
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G19" s="7" t="inlineStr">
@@ -1687,6 +1714,7 @@
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="7" t="n">
@@ -1699,12 +1727,12 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>Bỏ các cột không cần thiết</t>
+          <t>Cửa hàng và Mã đơn ở 2 cột đầu, có ô tìm kiếm</t>
         </is>
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Cột 'Ngày đi' tự đặt khi PD scan; giá lẻ gộp vào Tổng tiền; người phụ trách suy ra từ cửa hàng — không cần cột riêng.</t>
+          <t>Search hoạt động trên cả Cửa hàng và Mã đơn.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -1728,6 +1756,7 @@
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="7" t="n">
@@ -1740,12 +1769,12 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Gộp Tracking + tình trạng nhãn + carrier vào 1 cột</t>
+          <t>Bỏ các cột không cần thiết</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Hiển thị: 'Chờ in nhãn' / 'Đang mua nhãn' / '&lt;carrier&gt;: &lt;số tracking&gt;'.</t>
+          <t>Cột 'Ngày đi' tự đặt khi PD scan; giá lẻ gộp vào Tổng tiền; người phụ trách suy ra từ cửa hàng — không cần cột riêng.</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -1755,7 +1784,7 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
@@ -1769,6 +1798,7 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="7" t="n">
@@ -1781,17 +1811,17 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>Ảnh sản phẩm trên mỗi đơn</t>
+          <t>Gộp Tracking + tình trạng nhãn + carrier vào 1 cột</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Ảnh thu nhỏ 128px; bấm vào để xem ảnh lớn.</t>
+          <t>Hiển thị: 'Chờ in nhãn' / 'Đang mua nhãn' / '&lt;carrier&gt;: &lt;số tracking&gt;'.</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -1810,6 +1840,7 @@
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
+      <c r="J22" s="7" t="inlineStr"/>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="7" t="n">
@@ -1822,22 +1853,22 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Chỉnh trực tiếp các cột thao tác</t>
+          <t>Ảnh sản phẩm trên mỗi đơn</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>BA chỉnh ngay trên dòng: Tracking, Carrier, Tình trạng nhãn, Trạng thái đơn, Ghi chú.</t>
+          <t>Ảnh thu nhỏ 128px; bấm vào để xem ảnh lớn.</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>BA, Marketing</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G23" s="7" t="inlineStr">
@@ -1851,6 +1882,7 @@
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="7" t="n">
@@ -1863,17 +1895,17 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Tô màu hàng theo loại đơn</t>
+          <t>Chỉnh trực tiếp các cột thao tác</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Số lượng ≥ 2 tô cam; trùng mã tô tím; đơn ưu tiên (Push) tô đỏ; đơn Amazon tô đỏ.</t>
+          <t>BA chỉnh ngay trên dòng: Tracking, Carrier, Tình trạng nhãn, Trạng thái đơn, Ghi chú.</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>BA, Marketing</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -1892,6 +1924,7 @@
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
+      <c r="J24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="7" t="n">
@@ -1904,17 +1937,17 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Nút Push đánh dấu đơn ưu tiên</t>
+          <t>Tô màu hàng theo loại đơn</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Marketing bấm Push, đơn được đánh dấu và tô đỏ; lịch sử ghi lại ai bấm và lúc nào. Đơn Amazon đặt cùng ngày tự động được Push.</t>
+          <t>Số lượng ≥ 2 tô cam; trùng mã tô tím; đơn ưu tiên (Push) tô đỏ; đơn Amazon tô đỏ.</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -1933,6 +1966,7 @@
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="7" t="n">
@@ -1945,12 +1979,12 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Cảnh báo đơn quá 2 ngày chưa duyệt file</t>
+          <t>Nút Push đánh dấu đơn ưu tiên</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Đơn quá 2 ngày chưa duyệt file thiết kế tô vàng và hiện cảnh báo.</t>
+          <t>Marketing bấm Push, đơn được đánh dấu và tô đỏ; lịch sử ghi lại ai bấm và lúc nào. Đơn Amazon đặt cùng ngày tự động được Push.</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -1960,7 +1994,7 @@
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G26" s="7" t="inlineStr">
@@ -1974,6 +2008,7 @@
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
+      <c r="J26" s="7" t="inlineStr"/>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="7" t="n">
@@ -1986,12 +2021,12 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Cột hạn ship</t>
+          <t>Cảnh báo đơn quá 2 ngày chưa duyệt file</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Hiển thị hạn ship mà Etsy yêu cầu; quá hạn tô đỏ.</t>
+          <t>Đơn quá 2 ngày chưa duyệt file thiết kế tô vàng và hiện cảnh báo.</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -2001,7 +2036,7 @@
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G27" s="7" t="inlineStr">
@@ -2015,6 +2050,7 @@
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="7" t="n">
@@ -2027,12 +2063,12 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Avatar người quản lý cửa hàng</t>
+          <t>Cột hạn ship</t>
         </is>
       </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Mỗi đơn có avatar/icon của người quản lý cửa hàng tương ứng.</t>
+          <t>Hiển thị hạn ship mà Etsy yêu cầu; quá hạn tô đỏ.</t>
         </is>
       </c>
       <c r="E28" s="6" t="inlineStr">
@@ -2042,7 +2078,7 @@
       </c>
       <c r="F28" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G28" s="7" t="inlineStr">
@@ -2056,6 +2092,7 @@
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
+      <c r="J28" s="7" t="inlineStr"/>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="7" t="n">
@@ -2068,12 +2105,12 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Popup thông báo các sự kiện đặc biệt</t>
+          <t>Avatar người quản lý cửa hàng</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Push, tạm dừng, đổi địa chỉ — popup hiện đến đúng người trong 10 giây.</t>
+          <t>Mỗi đơn có avatar/icon của người quản lý cửa hàng tương ứng.</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2097,6 +2134,7 @@
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
+      <c r="J29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="7" t="n">
@@ -2109,22 +2147,22 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Trường 'Ghi chú Marketing' trên đơn</t>
+          <t>Popup thông báo các sự kiện đặc biệt</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
         <is>
-          <t>Tách riêng với 'Ghi chú đơn' để Marketing ghi yêu cầu custom của khách.</t>
+          <t>Push, tạm dừng, đổi địa chỉ — popup hiện đến đúng người trong 10 giây.</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G30" s="7" t="inlineStr">
@@ -2138,6 +2176,7 @@
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
+      <c r="J30" s="7" t="inlineStr"/>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="7" t="n">
@@ -2150,17 +2189,17 @@
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Lịch sử thay đổi trạng thái đơn</t>
+          <t>Trường 'Ghi chú Marketing' trên đơn</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Tab Lịch sử: ai đổi, lúc nào, từ giá trị nào sang giá trị nào.</t>
+          <t>Tách riêng với 'Ghi chú đơn' để Marketing ghi yêu cầu custom của khách.</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>BA, Marketing</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
@@ -2179,6 +2218,7 @@
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr"/>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="7" t="n">
@@ -2191,22 +2231,22 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>BA tự phân loại lại sản phẩm</t>
+          <t>Lịch sử thay đổi trạng thái đơn</t>
         </is>
       </c>
       <c r="D32" s="6" t="inlineStr">
         <is>
-          <t>BA có thể chỉnh phân loại sản phẩm tự động khi cần.</t>
+          <t>Tab Lịch sử: ai đổi, lúc nào, từ giá trị nào sang giá trị nào.</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BA, Marketing</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G32" s="7" t="inlineStr">
@@ -2220,6 +2260,7 @@
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr"/>
+      <c r="J32" s="7" t="inlineStr"/>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="7" t="n">
@@ -2232,22 +2273,22 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>Nhãn trạng thái file thiết kế trên mỗi dòng đơn</t>
+          <t>BA tự phân loại lại sản phẩm</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Mỗi dòng đơn hiện nhãn: chờ duyệt / đã duyệt / cần chỉnh sửa. Bấm vào để mở file.</t>
+          <t>BA có thể chỉnh phân loại sản phẩm tự động khi cần.</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>BA, Marketing</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G33" s="7" t="inlineStr">
@@ -2261,6 +2302,7 @@
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
+      <c r="J33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="7" t="n">
@@ -2268,27 +2310,27 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>4. Bảng điều khiển Vận chuyển</t>
+          <t>3. Bảng điều khiển Đơn hàng</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Trang Tracking riêng (không phải bộ lọc Đơn hàng)</t>
+          <t>Nhãn trạng thái file thiết kế trên mỗi dòng đơn</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Menu 'Tracking' mở ra trang riêng, có 13 cột phục vụ BA xử lý vận chuyển.</t>
+          <t>Mỗi dòng đơn hiện nhãn: chờ duyệt / đã duyệt / cần chỉnh sửa. Bấm vào để mở file.</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BA, Marketing</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G34" s="7" t="inlineStr">
@@ -2302,6 +2344,7 @@
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
+      <c r="J34" s="7" t="inlineStr"/>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="7" t="n">
@@ -2309,17 +2352,17 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>4. Bảng điều khiển Vận chuyển</t>
+          <t>3. Bảng điều khiển Đơn hàng</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>13 cột phục vụ vận chuyển</t>
+          <t>Bảng điều khiển dạng dòng sản phẩm (theo từng sản phẩm trong đơn)</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Mã đơn, Tracking, Carrier, Tình trạng, Loại sản phẩm, Số lượng, Tên người nhận, Địa chỉ 1-2, Thành phố, Bang, Mã ZIP, Quốc gia.</t>
+          <t>Bảng điều khiển Đơn hàng có chế độ xem theo từng dòng sản phẩm thay vì cả đơn — BA thấy ngay 34 cột thông tin Marketing đang dùng trên Excel (mã đơn, ảnh, chú thích cá nhân hoá, kích thước, số lượng, ngày hứa giao, người phụ trách...). Tất cả thao tác sửa, lọc, sắp xếp đều hoạt động ở mức dòng sản phẩm.</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -2343,6 +2386,7 @@
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
+      <c r="J35" s="7" t="inlineStr"/>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="7" t="n">
@@ -2355,12 +2399,12 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>Xuất Excel theo bộ lọc đang xem</t>
+          <t>Trang Tracking riêng (không phải bộ lọc Đơn hàng)</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Tải ra Excel đúng các đơn đang lọc trên màn hình.</t>
+          <t>Menu 'Tracking' mở ra trang riêng, có 13 cột phục vụ BA xử lý vận chuyển.</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
@@ -2370,7 +2414,7 @@
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G36" s="7" t="inlineStr">
@@ -2384,6 +2428,7 @@
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
+      <c r="J36" s="7" t="inlineStr"/>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="7" t="n">
@@ -2396,12 +2441,12 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Đổi trạng thái nhãn hàng loạt</t>
+          <t>13 cột phục vụ vận chuyển</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Chọn nhiều đơn cùng lúc và đổi từ 'Chờ in nhãn' sang 'Đang mua nhãn' chỉ với 1 thao tác.</t>
+          <t>Mã đơn, Tracking, Carrier, Tình trạng, Loại sản phẩm, Số lượng, Tên người nhận, Địa chỉ 1-2, Thành phố, Bang, Mã ZIP, Quốc gia.</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
@@ -2411,7 +2456,7 @@
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G37" s="7" t="inlineStr">
@@ -2425,6 +2470,7 @@
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
+      <c r="J37" s="7" t="inlineStr"/>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="7" t="n">
@@ -2437,12 +2483,12 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Ô tìm kiếm nhanh</t>
+          <t>Xuất Excel theo bộ lọc đang xem</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Tìm theo tracking, mã đơn hoặc tên khách ngay trên đầu trang.</t>
+          <t>Tải ra Excel đúng các đơn đang lọc trên màn hình.</t>
         </is>
       </c>
       <c r="E38" s="6" t="inlineStr">
@@ -2466,6 +2512,7 @@
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr"/>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="7" t="n">
@@ -2478,12 +2525,12 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Đồng bộ thay đổi sang Bảng điều khiển Đơn hàng</t>
+          <t>Đổi trạng thái nhãn hàng loạt</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Mọi cập nhật phản ánh sang bảng Đơn hàng trong vòng 5 giây.</t>
+          <t>Chọn nhiều đơn cùng lúc và đổi từ 'Chờ in nhãn' sang 'Đang mua nhãn' chỉ với 1 thao tác.</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
@@ -2493,7 +2540,7 @@
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G39" s="7" t="inlineStr">
@@ -2507,6 +2554,7 @@
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr"/>
     </row>
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="7" t="n">
@@ -2519,12 +2567,12 @@
       </c>
       <c r="C40" s="6" t="inlineStr">
         <is>
-          <t>Khoá thao tác mua nhãn khi đang chờ duyệt đổi địa chỉ</t>
+          <t>Ô tìm kiếm nhanh</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Vô hiệu nút 'Mua nhãn' và hiện cảnh báo khi đơn đang chờ duyệt đổi địa chỉ — tránh in nhãn sai địa chỉ.</t>
+          <t>Tìm theo tracking, mã đơn hoặc tên khách ngay trên đầu trang.</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
@@ -2534,7 +2582,7 @@
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G40" s="7" t="inlineStr">
@@ -2548,6 +2596,7 @@
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
+      <c r="J40" s="7" t="inlineStr"/>
     </row>
     <row r="41" ht="48" customHeight="1">
       <c r="A41" s="7" t="n">
@@ -2560,27 +2609,27 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Hiển thị tình trạng tracking thực tế (in-transit, delivered, returned)</t>
+          <t>Đồng bộ thay đổi sang Bảng điều khiển Đơn hàng</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Lấy tình trạng từ carrier (USPS, UniUni, YunExpress) và cập nhật lên màn hình theo thời gian thực.</t>
+          <t>Mọi cập nhật phản ánh sang bảng Đơn hàng trong vòng 5 giây.</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G41" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
@@ -2589,6 +2638,7 @@
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
+      <c r="J41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="7" t="n">
@@ -2596,17 +2646,17 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>5. Bảng điều khiển Sản xuất</t>
+          <t>4. Bảng điều khiển Vận chuyển</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Đặt tên 'Bảng điều khiển Sản xuất'</t>
+          <t>Khoá thao tác mua nhãn khi đang chờ duyệt đổi địa chỉ</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>BA và Sản xuất cùng dùng; bao gồm cả đơn Việt Nam và đơn Mỹ.</t>
+          <t>Vô hiệu nút 'Mua nhãn' và hiện cảnh báo khi đơn đang chờ duyệt đổi địa chỉ — tránh in nhãn sai địa chỉ.</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
@@ -2616,7 +2666,7 @@
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G42" s="7" t="inlineStr">
@@ -2630,6 +2680,7 @@
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
+      <c r="J42" s="7" t="inlineStr"/>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="7" t="n">
@@ -2637,32 +2688,32 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>5. Bảng điều khiển Sản xuất</t>
+          <t>4. Bảng điều khiển Vận chuyển</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Bộ cột phục vụ sản xuất</t>
+          <t>Hiển thị tình trạng tracking thực tế (in-transit, delivered, returned)</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Ngày duyệt file, Tải file, Tình trạng, Ghi chú, Ảnh, Lời nhắn quà tặng, Cá nhân hoá, Loại sản phẩm, Lựa chọn, Số lượng, Mã đơn, Cửa hàng, Tên khách, Địa chỉ, Dịch vụ vận chuyển, Ngày đặt, Ngày đi, Scan, Thống kê tự động.</t>
+          <t>Lấy tình trạng từ carrier (USPS, UniUni, YunExpress) và cập nhật lên màn hình theo thời gian thực.</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G43" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H43" s="7" t="inlineStr">
@@ -2671,6 +2722,7 @@
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
+      <c r="J43" s="7" t="inlineStr"/>
     </row>
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="7" t="n">
@@ -2678,27 +2730,27 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>5. Bảng điều khiển Sản xuất</t>
+          <t>4. Bảng điều khiển Vận chuyển</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Toàn bộ phòng ban xem trên CÙNG MỘT MÀN HÌNH</t>
+          <t>Trạng thái nhãn vận chuyển có ảnh minh hoạ</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Tất cả phòng ban xem chung một bảng (không phải tách 3 sheet như cách làm cũ). Phòng ban nào quan tâm thì lọc theo cột tình trạng / pipeline.</t>
+          <t>Khi BA chọn trạng thái cho nhãn vận chuyển (Đã in, Đã dán, Đã giao bưu cục, ...), danh sách tuỳ chọn hiển thị kèm ảnh thực tế của nhãn ở mỗi trạng thái — giúp BA nhận diện nhanh và giảm sai sót. Admin có thể thêm/sửa trạng thái và ảnh trong phần Cài đặt mà không cần lập trình viên.</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>BA, Sản xuất</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G44" s="7" t="inlineStr">
@@ -2711,11 +2763,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi của Owner</t>
-        </is>
-      </c>
+      <c r="I44" s="6" t="inlineStr"/>
+      <c r="J44" s="7" t="inlineStr"/>
     </row>
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="7" t="n">
@@ -2728,22 +2777,22 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Cột pipeline-state (giai đoạn sản xuất hiện tại)</t>
+          <t>Đặt tên 'Bảng điều khiển Sản xuất'</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Mỗi đơn hiển thị giai đoạn sản xuất hiện tại với màu của giai đoạn đó. Tên và ý nghĩa giai đoạn do admin tự cấu hình tại runtime, không cần lập trình.</t>
+          <t>BA và Sản xuất cùng dùng; bao gồm cả đơn Việt Nam và đơn Mỹ.</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G45" s="7" t="inlineStr">
@@ -2757,6 +2806,7 @@
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
+      <c r="J45" s="7" t="inlineStr"/>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="7" t="n">
@@ -2769,12 +2819,12 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Gán nhóm phụ trách cho từng giai đoạn</t>
+          <t>Bộ cột phục vụ sản xuất</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Mỗi giai đoạn sản xuất có thể gán mặc định cho một nhóm phụ trách. Có thể đổi cho từng đơn cụ thể khi cần.</t>
+          <t>Ngày duyệt file, Tải file, Tình trạng, Ghi chú, Ảnh, Lời nhắn quà tặng, Cá nhân hoá, Loại sản phẩm, Lựa chọn, Số lượng, Mã đơn, Cửa hàng, Tên khách, Địa chỉ, Dịch vụ vận chuyển, Ngày đặt, Ngày đi, Scan, Thống kê tự động.</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
@@ -2798,6 +2848,7 @@
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr"/>
+      <c r="J46" s="7" t="inlineStr"/>
     </row>
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="7" t="n">
@@ -2810,22 +2861,22 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Hiển thị ảnh thiết kế và bản preview</t>
+          <t>Toàn bộ phòng ban xem trên CÙNG MỘT MÀN HÌNH</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Mỗi dòng đơn có 2 ảnh thu nhỏ: file thiết kế gốc và bản preview gửi khách.</t>
+          <t>Tất cả phòng ban xem chung một bảng (không phải tách 3 sheet như cách làm cũ). Phòng ban nào quan tâm thì lọc theo cột tình trạng / pipeline.</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G47" s="7" t="inlineStr">
@@ -2838,7 +2889,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr"/>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi của Owner</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr"/>
     </row>
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="7" t="n">
@@ -2851,12 +2907,12 @@
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Widget thống kê đơn</t>
+          <t>Cột pipeline-state (giai đoạn sản xuất hiện tại)</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Đếm theo giai đoạn sản xuất, lựa chọn, loại sản phẩm, số lượng.</t>
+          <t>Mỗi đơn hiển thị giai đoạn sản xuất hiện tại với màu của giai đoạn đó. Tên và ý nghĩa giai đoạn do admin tự cấu hình tại runtime, không cần lập trình.</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
@@ -2866,7 +2922,7 @@
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G48" s="7" t="inlineStr">
@@ -2880,6 +2936,7 @@
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
+      <c r="J48" s="7" t="inlineStr"/>
     </row>
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="7" t="n">
@@ -2892,22 +2949,22 @@
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Scan barcode để chốt đơn hoàn thành</t>
+          <t>Gán nhóm phụ trách cho từng giai đoạn</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>PD scan barcode, đơn tự nhảy về giai đoạn cuối được đánh dấu 'hoàn tất'; ngày ship tự đặt; lịch sử ghi lại ai scan và lúc nào.</t>
+          <t>Mỗi giai đoạn sản xuất có thể gán mặc định cho một nhóm phụ trách. Có thể đổi cho từng đơn cụ thể khi cần.</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất, BA</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G49" s="7" t="inlineStr">
@@ -2921,6 +2978,7 @@
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
+      <c r="J49" s="7" t="inlineStr"/>
     </row>
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="7" t="n">
@@ -2933,22 +2991,22 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Lịch sử các thay đổi giai đoạn sản xuất</t>
+          <t>Hiển thị ảnh thiết kế và bản preview</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Mọi thay đổi cấu trúc pipeline, đổi tên giai đoạn, đổi nhóm phụ trách, hoặc đơn nhảy giai đoạn đều được ghi vào sổ lịch sử để truy vết.</t>
+          <t>Mỗi dòng đơn có 2 ảnh thu nhỏ: file thiết kế gốc và bản preview gửi khách.</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G50" s="7" t="inlineStr">
@@ -2962,6 +3020,7 @@
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
+      <c r="J50" s="7" t="inlineStr"/>
     </row>
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="7" t="n">
@@ -2969,27 +3028,27 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
+          <t>5. Bảng điều khiển Sản xuất</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Cho phép upload lại file thiết kế kích thước lớn</t>
+          <t>Widget thống kê đơn</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Designer có thể upload file lớn (ví dụ 150MB) lên Google Drive; có thể xoá và up lại; bản cũ vẫn được lưu để truy vết.</t>
+          <t>Đếm theo giai đoạn sản xuất, lựa chọn, loại sản phẩm, số lượng.</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G51" s="7" t="inlineStr">
@@ -3003,6 +3062,7 @@
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
+      <c r="J51" s="7" t="inlineStr"/>
     </row>
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="7" t="n">
@@ -3010,27 +3070,27 @@
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
+          <t>5. Bảng điều khiển Sản xuất</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>Quy trình duyệt file thiết kế</t>
+          <t>Scan barcode để chốt đơn hoàn thành</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>File thiết kế đi qua 3 trạng thái: Chờ duyệt → Đã duyệt / Cần chỉnh sửa (phải nhập lý do). Lưu lại ai duyệt và thời điểm duyệt.</t>
+          <t>PD scan barcode, đơn tự nhảy về giai đoạn cuối được đánh dấu 'hoàn tất'; ngày ship tự đặt; lịch sử ghi lại ai scan và lúc nào.</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>Sản xuất, BA</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G52" s="7" t="inlineStr">
@@ -3044,6 +3104,7 @@
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
+      <c r="J52" s="7" t="inlineStr"/>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="7" t="n">
@@ -3051,27 +3112,27 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
+          <t>5. Bảng điều khiển Sản xuất</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Hàng đợi thiết kế dạng kanban 3 cột</t>
+          <t>Lịch sử các thay đổi giai đoạn sản xuất</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Designer và BA kéo-thả hoặc click để chuyển file giữa các trạng thái duyệt.</t>
+          <t>Mọi thay đổi cấu trúc pipeline, đổi tên giai đoạn, đổi nhóm phụ trách, hoặc đơn nhảy giai đoạn đều được ghi vào sổ lịch sử để truy vết.</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G53" s="7" t="inlineStr">
@@ -3085,6 +3146,7 @@
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
+      <c r="J53" s="7" t="inlineStr"/>
     </row>
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="7" t="n">
@@ -3097,12 +3159,12 @@
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Quy trình duyệt đổi địa chỉ giao hàng</t>
+          <t>Cho phép upload lại file thiết kế kích thước lớn</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Marketing không sửa địa chỉ trực tiếp. Phải tạo yêu cầu đổi → BA duyệt hoặc từ chối → rồi mới được sửa.</t>
+          <t>Designer có thể upload file lớn (ví dụ 150MB) lên Google Drive; có thể xoá và up lại; bản cũ vẫn được lưu để truy vết.</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
@@ -3126,6 +3188,7 @@
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
+      <c r="J54" s="7" t="inlineStr"/>
     </row>
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="7" t="n">
@@ -3138,17 +3201,17 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Khoá mua nhãn khi đang chờ duyệt đổi địa chỉ</t>
+          <t>Quy trình duyệt file thiết kế</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Vô hiệu nút Mua nhãn và hiện cảnh báo trên Bảng Vận chuyển.</t>
+          <t>File thiết kế đi qua 3 trạng thái: Chờ duyệt → Đã duyệt / Cần chỉnh sửa (phải nhập lý do). Lưu lại ai duyệt và thời điểm duyệt.</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -3167,6 +3230,7 @@
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
+      <c r="J55" s="7" t="inlineStr"/>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="7" t="n">
@@ -3179,12 +3243,12 @@
       </c>
       <c r="C56" s="6" t="inlineStr">
         <is>
-          <t>Tạo ticket đổi/hoàn tiền từ trang chi tiết đơn</t>
+          <t>Hàng đợi thiết kế dạng kanban 3 cột</t>
         </is>
       </c>
       <c r="D56" s="6" t="inlineStr">
         <is>
-          <t>Form đơn có nút 'Tạo ticket'; Marketing nhập lý do và ảnh; chọn loại: đổi hàng, hoàn tiền, hoặc giảm giá; gửi BA duyệt.</t>
+          <t>Designer và BA kéo-thả hoặc click để chuyển file giữa các trạng thái duyệt.</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
@@ -3199,7 +3263,7 @@
       </c>
       <c r="G56" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H56" s="7" t="inlineStr">
@@ -3208,6 +3272,7 @@
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
+      <c r="J56" s="7" t="inlineStr"/>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="7" t="n">
@@ -3220,12 +3285,12 @@
       </c>
       <c r="C57" s="6" t="inlineStr">
         <is>
-          <t>BA duyệt ticket → hệ thống tự xử lý</t>
+          <t>Quy trình duyệt đổi địa chỉ giao hàng</t>
         </is>
       </c>
       <c r="D57" s="6" t="inlineStr">
         <is>
-          <t>Hoàn tiền sinh credit note; đổi hàng tạo đơn mới link đơn cũ; giảm giá ghi nhận giảm trên đơn.</t>
+          <t>Marketing không sửa địa chỉ trực tiếp. Phải tạo yêu cầu đổi → BA duyệt hoặc từ chối → rồi mới được sửa.</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
@@ -3235,12 +3300,12 @@
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G57" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H57" s="7" t="inlineStr">
@@ -3249,6 +3314,7 @@
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
+      <c r="J57" s="7" t="inlineStr"/>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="7" t="n">
@@ -3261,12 +3327,12 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>Lịch sử ticket trên trang đơn</t>
+          <t>Khoá mua nhãn khi đang chờ duyệt đổi địa chỉ</t>
         </is>
       </c>
       <c r="D58" s="6" t="inlineStr">
         <is>
-          <t>Tab 'Lịch sử' hiển thị toàn bộ thao tác của ticket trên đơn đó.</t>
+          <t>Vô hiệu nút Mua nhãn và hiện cảnh báo trên Bảng Vận chuyển.</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
@@ -3276,12 +3342,12 @@
       </c>
       <c r="F58" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G58" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H58" s="7" t="inlineStr">
@@ -3290,6 +3356,7 @@
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
+      <c r="J58" s="7" t="inlineStr"/>
     </row>
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="7" t="n">
@@ -3297,32 +3364,32 @@
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>7. Nhập tracking &amp; giao đối tác</t>
+          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
         </is>
       </c>
       <c r="C59" s="6" t="inlineStr">
         <is>
-          <t>Nhập tracking từ file Excel logistics (GKE)</t>
+          <t>Tạo ticket đổi/hoàn tiền từ trang chi tiết đơn</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
         <is>
-          <t>Tải Excel chuẩn GKE lên; hệ thống khớp Mã đơn rồi tự điền tracking và carrier. Hàng không khớp được liệt kê cho BA xử lý tay.</t>
+          <t>Form đơn có nút 'Tạo ticket'; Marketing nhập lý do và ảnh; chọn loại: đổi hàng, hoàn tiền, hoặc giảm giá; gửi BA duyệt.</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>BA, Logistics</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G59" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H59" s="7" t="inlineStr">
@@ -3330,11 +3397,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: thay vì copy tay từ file logistics sang Google Excel</t>
-        </is>
-      </c>
+      <c r="I59" s="6" t="inlineStr"/>
+      <c r="J59" s="7" t="inlineStr"/>
     </row>
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="7" t="n">
@@ -3342,32 +3406,32 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>7. Nhập tracking &amp; giao đối tác</t>
+          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
         </is>
       </c>
       <c r="C60" s="6" t="inlineStr">
         <is>
-          <t>Tự nhận diện carrier từ số tracking</t>
+          <t>BA duyệt ticket → hệ thống tự xử lý</t>
         </is>
       </c>
       <c r="D60" s="6" t="inlineStr">
         <is>
-          <t>20-22 chữ số → USPS; bắt đầu 'UU' → UniUni; bắt đầu 'YT' → YunExpress; còn lại → 'Khác'.</t>
+          <t>Hoàn tiền sinh credit note; đổi hàng tạo đơn mới link đơn cũ; giảm giá ghi nhận giảm trên đơn.</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Logistics</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G60" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H60" s="7" t="inlineStr">
@@ -3376,6 +3440,7 @@
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
+      <c r="J60" s="7" t="inlineStr"/>
     </row>
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="7" t="n">
@@ -3383,32 +3448,32 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>7. Nhập tracking &amp; giao đối tác</t>
+          <t>6. Quy trình duyệt (file thiết kế / địa chỉ / ticket)</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>Xử lý đơn '-replace' và lưu URL nhãn / mã QR</t>
+          <t>Lịch sử ticket trên trang đơn</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Đơn có hậu tố '-replace' tự động link đơn gốc. URL nhãn và mã QR lưu trên đơn.</t>
+          <t>Tab 'Lịch sử' hiển thị toàn bộ thao tác của ticket trên đơn đó.</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>BA, Logistics</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G61" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H61" s="7" t="inlineStr">
@@ -3417,6 +3482,7 @@
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
+      <c r="J61" s="7" t="inlineStr"/>
     </row>
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="7" t="n">
@@ -3429,22 +3495,22 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Báo cáo nhập tracking (đã khớp / chưa khớp)</t>
+          <t>Nhập tracking từ file Excel logistics (GKE)</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Sau khi nhập, hiện wizard tóm tắt và cho phép xem chi tiết các dòng lỗi.</t>
+          <t>Tải Excel chuẩn GKE lên; hệ thống khớp Mã đơn rồi tự điền tracking và carrier. Hàng không khớp được liệt kê cho BA xử lý tay.</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BA, Logistics</t>
         </is>
       </c>
       <c r="F62" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G62" s="7" t="inlineStr">
@@ -3457,7 +3523,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I62" s="6" t="inlineStr"/>
+      <c r="I62" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: thay vì copy tay từ file logistics sang Google Excel</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr"/>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="7" t="n">
@@ -3470,17 +3541,17 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Kết nối Gearment và đẩy đơn</t>
+          <t>Tự nhận diện carrier từ số tracking</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Cấu hình Gearment 1 lần; BA bấm 'Push to Gearment' để đẩy đơn kèm file thiết kế.</t>
+          <t>20-22 chữ số → USPS; bắt đầu 'UU' → UniUni; bắt đầu 'YT' → YunExpress; còn lại → 'Khác'.</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án, BA</t>
+          <t>Logistics</t>
         </is>
       </c>
       <c r="F63" s="7" t="inlineStr">
@@ -3490,7 +3561,7 @@
       </c>
       <c r="G63" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
@@ -3499,6 +3570,7 @@
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr"/>
     </row>
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="7" t="n">
@@ -3511,27 +3583,27 @@
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Quy trình Gearment 4 bước</t>
+          <t>Xử lý đơn '-replace' và lưu URL nhãn / mã QR</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Nháp → báo giá → BA duyệt → xác nhận đặt sản xuất.</t>
+          <t>Đơn có hậu tố '-replace' tự động link đơn gốc. URL nhãn và mã QR lưu trên đơn.</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>BA, Logistics</t>
         </is>
       </c>
       <c r="F64" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G64" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H64" s="7" t="inlineStr">
@@ -3540,6 +3612,7 @@
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
+      <c r="J64" s="7" t="inlineStr"/>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="7" t="n">
@@ -3552,27 +3625,27 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Nhận tracking và tình trạng từ Gearment</t>
+          <t>Báo cáo nhập tracking (đã khớp / chưa khớp)</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống nhận thông báo từ Gearment hoặc tự kéo theo lịch để cập nhật đơn, rồi đẩy tracking lên Etsy nếu Marketing đã bật tự đẩy.</t>
+          <t>Sau khi nhập, hiện wizard tóm tắt và cho phép xem chi tiết các dòng lỗi.</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>BA, Marketing</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F65" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G65" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
@@ -3581,6 +3654,7 @@
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
+      <c r="J65" s="7" t="inlineStr"/>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="7" t="n">
@@ -3593,22 +3667,22 @@
       </c>
       <c r="C66" s="6" t="inlineStr">
         <is>
-          <t>Xử lý lỗi và thử lại tự động</t>
+          <t>Kết nối Gearment và đẩy đơn</t>
         </is>
       </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Mỗi đơn thử tối đa 3 lần; nếu vẫn lỗi sẽ ghi nhật ký và cảnh báo admin.</t>
+          <t>Cấu hình Gearment 1 lần; BA bấm 'Push to Gearment' để đẩy đơn kèm file thiết kế.</t>
         </is>
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>Chủ dự án, BA</t>
         </is>
       </c>
       <c r="F66" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G66" s="7" t="inlineStr">
@@ -3622,6 +3696,7 @@
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr"/>
+      <c r="J66" s="7" t="inlineStr"/>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="7" t="n">
@@ -3634,12 +3709,12 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Chính sách huỷ đơn nháp ở Gearment khi rework</t>
+          <t>Quy trình Gearment 4 bước</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Khi Marketing yêu cầu làm lại đơn (giai đoạn 'Sửa'), đơn nháp/báo giá cũ phía Gearment phải được huỷ hoặc tự hết hạn.</t>
+          <t>Nháp → báo giá → BA duyệt → xác nhận đặt sản xuất.</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
@@ -3663,6 +3738,7 @@
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
+      <c r="J67" s="7" t="inlineStr"/>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="7" t="n">
@@ -3670,22 +3746,22 @@
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>8. Quản lý file thiết kế</t>
+          <t>7. Nhập tracking &amp; giao đối tác</t>
         </is>
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>Một lần upload — gửi đến nhiều nơi</t>
+          <t>Nhận tracking và tình trạng từ Gearment</t>
         </is>
       </c>
       <c r="D68" s="6" t="inlineStr">
         <is>
-          <t>BA upload file 1 lần; hệ thống lưu file và checksum. Có thể gửi sang nhiều nơi nhận (Marketing duyệt, PD in, đối tác sản xuất) mà không cần upload lại.</t>
+          <t>Hệ thống nhận thông báo từ Gearment hoặc tự kéo theo lịch để cập nhật đơn, rồi đẩy tracking lên Etsy nếu Marketing đã bật tự đẩy.</t>
         </is>
       </c>
       <c r="E68" s="6" t="inlineStr">
         <is>
-          <t>Marketing, BA, Sản xuất</t>
+          <t>BA, Marketing</t>
         </is>
       </c>
       <c r="F68" s="7" t="inlineStr">
@@ -3695,7 +3771,7 @@
       </c>
       <c r="G68" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
@@ -3703,11 +3779,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I68" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: file 8MB không gửi được Discord, hay bị thất lạc, mất thời gian tải lên-tải xuống nhiều lần</t>
-        </is>
-      </c>
+      <c r="I68" s="6" t="inlineStr"/>
+      <c r="J68" s="7" t="inlineStr"/>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="7" t="n">
@@ -3715,32 +3788,32 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>8. Quản lý file thiết kế</t>
+          <t>7. Nhập tracking &amp; giao đối tác</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
         <is>
-          <t>Theo dõi tình trạng nhận file của từng nơi</t>
+          <t>Xử lý lỗi và thử lại tự động</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Mỗi lần gửi file đi đâu đều ghi nhận: chờ gửi / đã gửi / đã xác nhận / lỗi và thời điểm tương ứng.</t>
+          <t>Mỗi đơn thử tối đa 3 lần; nếu vẫn lỗi sẽ ghi nhật ký và cảnh báo admin.</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F69" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
@@ -3749,6 +3822,7 @@
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr"/>
+      <c r="J69" s="7" t="inlineStr"/>
     </row>
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="7" t="n">
@@ -3756,32 +3830,32 @@
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>8. Quản lý file thiết kế</t>
+          <t>7. Nhập tracking &amp; giao đối tác</t>
         </is>
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>Wizard tải hàng loạt file đã duyệt theo khổ A4</t>
+          <t>Chính sách huỷ đơn nháp ở Gearment khi rework</t>
         </is>
       </c>
       <c r="D70" s="6" t="inlineStr">
         <is>
-          <t>PD chọn nhiều file đã duyệt cùng lúc, hệ thống dàn thành PDF khổ A4 và lưu cache 24h để PD in.</t>
+          <t>Khi Marketing yêu cầu làm lại đơn (giai đoạn 'Sửa'), đơn nháp/báo giá cũ phía Gearment phải được huỷ hoặc tự hết hạn.</t>
         </is>
       </c>
       <c r="E70" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F70" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 1</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H70" s="7" t="inlineStr">
@@ -3789,11 +3863,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I70" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: PD mất nhiều thời gian search mã đơn, download file, sắp lên Photoshop</t>
-        </is>
-      </c>
+      <c r="I70" s="6" t="inlineStr"/>
+      <c r="J70" s="7" t="inlineStr"/>
     </row>
     <row r="71" ht="48" customHeight="1">
       <c r="A71" s="7" t="n">
@@ -3806,22 +3877,22 @@
       </c>
       <c r="C71" s="6" t="inlineStr">
         <is>
-          <t>Lưu trữ chính trên Google Drive, có hàng đợi an toàn khi lỗi</t>
+          <t>Một lần upload — gửi đến nhiều nơi</t>
         </is>
       </c>
       <c r="D71" s="6" t="inlineStr">
         <is>
-          <t>Khi Google Drive gặp sự cố, hệ thống không chuyển ngầm sang Discord — thay vào đó đưa file vào hàng đợi và cảnh báo. Discord vẫn được giữ làm kênh thủ công khẩn cấp.</t>
+          <t>BA upload file 1 lần; hệ thống lưu file và checksum. Có thể gửi sang nhiều nơi nhận (Marketing duyệt, PD in, đối tác sản xuất) mà không cần upload lại.</t>
         </is>
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Marketing, BA, Sản xuất</t>
         </is>
       </c>
       <c r="F71" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G71" s="7" t="inlineStr">
@@ -3834,7 +3905,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I71" s="6" t="inlineStr"/>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: file 8MB không gửi được Discord, hay bị thất lạc, mất thời gian tải lên-tải xuống nhiều lần</t>
+        </is>
+      </c>
+      <c r="J71" s="7" t="inlineStr"/>
     </row>
     <row r="72" ht="48" customHeight="1">
       <c r="A72" s="7" t="n">
@@ -3847,22 +3923,22 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Upload lại sau khi 'Cần chỉnh sửa' tạo bản version mới</t>
+          <t>Theo dõi tình trạng nhận file của từng nơi</t>
         </is>
       </c>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>File bị từ chối ở trạng thái 'cần chỉnh sửa'. Bản upload mới được lưu là phiên bản tiếp theo (link tới bản cũ) để có thể đo tỷ lệ duyệt lần đầu.</t>
+          <t>Mỗi lần gửi file đi đâu đều ghi nhận: chờ gửi / đã gửi / đã xác nhận / lỗi và thời điểm tương ứng.</t>
         </is>
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>BA, Sản xuất</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F72" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G72" s="7" t="inlineStr">
@@ -3876,6 +3952,7 @@
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
+      <c r="J72" s="7" t="inlineStr"/>
     </row>
     <row r="73" ht="48" customHeight="1">
       <c r="A73" s="7" t="n">
@@ -3888,17 +3965,17 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>Cảnh báo khi 'gửi file' bị treo &gt; 2 giờ</t>
+          <t>Wizard tải hàng loạt file đã duyệt theo khổ A4</t>
         </is>
       </c>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Nếu thao tác gửi file (cấp quyền Google Drive, đẩy sang đối tác) chưa xong sau 2 giờ, đơn nổi cảnh báo trên Bảng Sản xuất.</t>
+          <t>PD chọn nhiều file đã duyệt cùng lúc, hệ thống dàn thành PDF khổ A4 và lưu cache 24h để PD in.</t>
         </is>
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất, BA</t>
+          <t>Sản xuất</t>
         </is>
       </c>
       <c r="F73" s="7" t="inlineStr">
@@ -3916,7 +3993,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I73" s="6" t="inlineStr"/>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: PD mất nhiều thời gian search mã đơn, download file, sắp lên Photoshop</t>
+        </is>
+      </c>
+      <c r="J73" s="7" t="inlineStr"/>
     </row>
     <row r="74" ht="48" customHeight="1">
       <c r="A74" s="7" t="n">
@@ -3929,12 +4011,12 @@
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Tự động gửi file thiết kế khi BA xác nhận đơn</t>
+          <t>Lưu trữ chính trên Google Drive, có hàng đợi an toàn khi lỗi</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Khi BA xác nhận đơn có file đã duyệt, hệ thống tự tạo các phiếu gửi file đến đúng nơi nhận và chạy nền để cấp quyền/gửi đi.</t>
+          <t>Khi Google Drive gặp sự cố, hệ thống không chuyển ngầm sang Discord — thay vào đó đưa file vào hàng đợi và cảnh báo. Discord vẫn được giữ làm kênh thủ công khẩn cấp.</t>
         </is>
       </c>
       <c r="E74" s="6" t="inlineStr">
@@ -3958,6 +4040,7 @@
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
+      <c r="J74" s="7" t="inlineStr"/>
     </row>
     <row r="75" ht="48" customHeight="1">
       <c r="A75" s="7" t="n">
@@ -3965,27 +4048,27 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>9. Pipeline sản xuất có thể cấu hình</t>
+          <t>8. Quản lý file thiết kế</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
         <is>
-          <t>Pipeline có thể tự định nghĩa (không cần lập trình)</t>
+          <t>Upload lại sau khi 'Cần chỉnh sửa' tạo bản version mới</t>
         </is>
       </c>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Admin tự đặt tên pipeline, thêm/sửa/xoá giai đoạn, đặt màu, đánh dấu giai đoạn bắt đầu/giai đoạn kết thúc.</t>
+          <t>File bị từ chối ở trạng thái 'cần chỉnh sửa'. Bản upload mới được lưu là phiên bản tiếp theo (link tới bản cũ) để có thể đo tỷ lệ duyệt lần đầu.</t>
         </is>
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án, Sản xuất</t>
+          <t>BA, Sản xuất</t>
         </is>
       </c>
       <c r="F75" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G75" s="7" t="inlineStr">
@@ -3999,6 +4082,7 @@
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr"/>
     </row>
     <row r="76" ht="48" customHeight="1">
       <c r="A76" s="7" t="n">
@@ -4006,27 +4090,27 @@
       </c>
       <c r="B76" s="6" t="inlineStr">
         <is>
-          <t>9. Pipeline sản xuất có thể cấu hình</t>
+          <t>8. Quản lý file thiết kế</t>
         </is>
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Mỗi sản phẩm/danh mục dùng pipeline phù hợp</t>
+          <t>Cảnh báo khi 'gửi file' bị treo &gt; 2 giờ</t>
         </is>
       </c>
       <c r="D76" s="6" t="inlineStr">
         <is>
-          <t>Sản phẩm chọn pipeline mặc định; nếu chưa, lấy theo danh mục; nếu vẫn chưa, dùng pipeline mặc định toàn hệ thống.</t>
+          <t>Nếu thao tác gửi file (cấp quyền Google Drive, đẩy sang đối tác) chưa xong sau 2 giờ, đơn nổi cảnh báo trên Bảng Sản xuất.</t>
         </is>
       </c>
       <c r="E76" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>Sản xuất, BA</t>
         </is>
       </c>
       <c r="F76" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -4040,6 +4124,7 @@
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr"/>
+      <c r="J76" s="7" t="inlineStr"/>
     </row>
     <row r="77" ht="48" customHeight="1">
       <c r="A77" s="7" t="n">
@@ -4047,17 +4132,17 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>9. Pipeline sản xuất có thể cấu hình</t>
+          <t>8. Quản lý file thiết kế</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
         <is>
-          <t>Đơn có nhiều sản phẩm khác pipeline — BA chọn pipeline</t>
+          <t>Tự động gửi file thiết kế khi BA xác nhận đơn</t>
         </is>
       </c>
       <c r="D77" s="6" t="inlineStr">
         <is>
-          <t>Khi đơn chứa nhiều sản phẩm thuộc nhiều pipeline, mặc định lấy pipeline của sản phẩm đầu tiên; UI cảnh báo để BA xác nhận lại.</t>
+          <t>Khi BA xác nhận đơn có file đã duyệt, hệ thống tự tạo các phiếu gửi file đến đúng nơi nhận và chạy nền để cấp quyền/gửi đi.</t>
         </is>
       </c>
       <c r="E77" s="6" t="inlineStr">
@@ -4081,6 +4166,7 @@
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr"/>
     </row>
     <row r="78" ht="48" customHeight="1">
       <c r="A78" s="7" t="n">
@@ -4093,17 +4179,17 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>Tự sao lưu phiên bản pipeline khi sửa lúc đang có đơn chạy</t>
+          <t>Pipeline có thể tự định nghĩa (không cần lập trình)</t>
         </is>
       </c>
       <c r="D78" s="6" t="inlineStr">
         <is>
-          <t>Khi pipeline đang được dùng bị sửa, hệ thống tạo phiên bản mới tự động; đơn cũ tiếp tục dùng phiên bản cũ; đơn mới dùng phiên bản mới.</t>
+          <t>Admin tự đặt tên pipeline, thêm/sửa/xoá giai đoạn, đặt màu, đánh dấu giai đoạn bắt đầu/giai đoạn kết thúc.</t>
         </is>
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>Chủ dự án, Sản xuất</t>
         </is>
       </c>
       <c r="F78" s="7" t="inlineStr">
@@ -4122,6 +4208,7 @@
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
+      <c r="J78" s="7" t="inlineStr"/>
     </row>
     <row r="79" ht="48" customHeight="1">
       <c r="A79" s="7" t="n">
@@ -4134,12 +4221,12 @@
       </c>
       <c r="C79" s="6" t="inlineStr">
         <is>
-          <t>Chính sách di chuyển giữa các giai đoạn</t>
+          <t>Mỗi sản phẩm/danh mục dùng pipeline phù hợp</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Mỗi pipeline chọn một trong các kiểu: theo sơ đồ chặt; theo sơ đồ nhưng admin được phá rào; tự do chuyển bất kỳ. Mặc định là sơ đồ với quyền admin phá rào.</t>
+          <t>Sản phẩm chọn pipeline mặc định; nếu chưa, lấy theo danh mục; nếu vẫn chưa, dùng pipeline mặc định toàn hệ thống.</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
@@ -4163,6 +4250,7 @@
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr"/>
+      <c r="J79" s="7" t="inlineStr"/>
     </row>
     <row r="80" ht="48" customHeight="1">
       <c r="A80" s="7" t="n">
@@ -4175,22 +4263,22 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>Bộ pipeline mẫu sẵn</t>
+          <t>Đơn có nhiều sản phẩm khác pipeline — BA chọn pipeline</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống ship sẵn 3 pipeline mẫu: 'Sản xuất nội bộ Việt Nam' (17 giai đoạn từ thực tế PD đang dùng), 'Gearment POD' (4 giai đoạn), 'Đa kỹ thuật pha trộn'.</t>
+          <t>Khi đơn chứa nhiều sản phẩm thuộc nhiều pipeline, mặc định lấy pipeline của sản phẩm đầu tiên; UI cảnh báo để BA xác nhận lại.</t>
         </is>
       </c>
       <c r="E80" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F80" s="7" t="inlineStr">
         <is>
-          <t>Cao</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G80" s="7" t="inlineStr">
@@ -4204,6 +4292,7 @@
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr"/>
+      <c r="J80" s="7" t="inlineStr"/>
     </row>
     <row r="81" ht="48" customHeight="1">
       <c r="A81" s="7" t="n">
@@ -4216,12 +4305,12 @@
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Sổ lịch sử pipeline duy nhất</t>
+          <t>Tự sao lưu phiên bản pipeline khi sửa lúc đang có đơn chạy</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Mọi thay đổi (sửa pipeline, đổi tên giai đoạn, đổi nhóm phụ trách, đơn chuyển giai đoạn) ghi vào cùng một sổ lịch sử để dễ truy vết.</t>
+          <t>Khi pipeline đang được dùng bị sửa, hệ thống tạo phiên bản mới tự động; đơn cũ tiếp tục dùng phiên bản cũ; đơn mới dùng phiên bản mới.</t>
         </is>
       </c>
       <c r="E81" s="6" t="inlineStr">
@@ -4245,6 +4334,7 @@
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
+      <c r="J81" s="7" t="inlineStr"/>
     </row>
     <row r="82" ht="48" customHeight="1">
       <c r="A82" s="7" t="n">
@@ -4257,27 +4347,27 @@
       </c>
       <c r="C82" s="6" t="inlineStr">
         <is>
-          <t>Trigger tự nhảy giai đoạn (giai đoạn 2)</t>
+          <t>Chính sách di chuyển giữa các giai đoạn</t>
         </is>
       </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống cho cấu hình trigger tự nhảy giai đoạn (khi thanh toán, khi duyệt thiết kế, khi nhập tracking) — bật ở giai đoạn 2.</t>
+          <t>Mỗi pipeline chọn một trong các kiểu: theo sơ đồ chặt; theo sơ đồ nhưng admin được phá rào; tự do chuyển bất kỳ. Mặc định là sơ đồ với quyền admin phá rào.</t>
         </is>
       </c>
       <c r="E82" s="6" t="inlineStr">
         <is>
-          <t>Marketing, BA, Sản xuất</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F82" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G82" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H82" s="7" t="inlineStr">
@@ -4286,6 +4376,7 @@
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
+      <c r="J82" s="7" t="inlineStr"/>
     </row>
     <row r="83" ht="48" customHeight="1">
       <c r="A83" s="7" t="n">
@@ -4293,32 +4384,32 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>10. Hộp thư khách hàng</t>
+          <t>9. Pipeline sản xuất có thể cấu hình</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
         <is>
-          <t>Tổng hợp tin nhắn khách 19 cửa hàng vào một chỗ</t>
+          <t>Bộ pipeline mẫu sẵn</t>
         </is>
       </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Hệ thống tự kéo lời nhắn của khách (buyer message) khi khách đặt hàng và hiển thị: (a) trên trang đơn; (b) trên trang 'Hộp thư khách hàng' để Marketing/BA tìm xuyên cửa hàng.</t>
+          <t>Hệ thống ship sẵn 3 pipeline mẫu: 'Sản xuất nội bộ Việt Nam' (17 giai đoạn từ thực tế PD đang dùng), 'Gearment POD' (4 giai đoạn), 'Đa kỹ thuật pha trộn'.</t>
         </is>
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F83" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G83" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H83" s="7" t="inlineStr">
@@ -4326,11 +4417,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I83" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: chưa có dashboard tổng hợp tin nhắn khách trong ngày</t>
-        </is>
-      </c>
+      <c r="I83" s="6" t="inlineStr"/>
+      <c r="J83" s="7" t="inlineStr"/>
     </row>
     <row r="84" ht="48" customHeight="1">
       <c r="A84" s="7" t="n">
@@ -4338,32 +4426,32 @@
       </c>
       <c r="B84" s="6" t="inlineStr">
         <is>
-          <t>11. Mở rộng giai đoạn 2-3</t>
+          <t>9. Pipeline sản xuất có thể cấu hình</t>
         </is>
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>Bảng kiểm soát giá (Pricing Audit) 25 cột</t>
+          <t>Sổ lịch sử pipeline duy nhất</t>
         </is>
       </c>
       <c r="D84" s="6" t="inlineStr">
         <is>
-          <t>RD nhập tay 6 cột (A-F), 19 cột còn lại tự lấy từ đơn. Hỗ trợ đa tiền tệ.</t>
+          <t>Mọi thay đổi (sửa pipeline, đổi tên giai đoạn, đổi nhóm phụ trách, đơn chuyển giai đoạn) ghi vào cùng một sổ lịch sử để dễ truy vết.</t>
         </is>
       </c>
       <c r="E84" s="6" t="inlineStr">
         <is>
-          <t>Kiểm soát giá</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F84" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Cao</t>
         </is>
       </c>
       <c r="G84" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 2</t>
+          <t>Giai đoạn 1</t>
         </is>
       </c>
       <c r="H84" s="7" t="inlineStr">
@@ -4372,6 +4460,7 @@
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
+      <c r="J84" s="7" t="inlineStr"/>
     </row>
     <row r="85" ht="48" customHeight="1">
       <c r="A85" s="7" t="n">
@@ -4379,27 +4468,27 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>11. Mở rộng giai đoạn 2-3</t>
+          <t>9. Pipeline sản xuất có thể cấu hình</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
         <is>
-          <t>Quy đổi giá đơn về EUR theo ngày đặt</t>
+          <t>Trigger tự nhảy giai đoạn (giai đoạn 2)</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Tự quy đổi USD/VND/CAD về EUR theo tỷ giá ngày đặt. Hiện 'Tổng tiền (EUR)'.</t>
+          <t>Hệ thống cho cấu hình trigger tự nhảy giai đoạn (khi thanh toán, khi duyệt thiết kế, khi nhập tracking) — bật ở giai đoạn 2.</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Kiểm soát giá</t>
+          <t>Marketing, BA, Sản xuất</t>
         </is>
       </c>
       <c r="F85" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G85" s="7" t="inlineStr">
@@ -4413,6 +4502,7 @@
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr"/>
+      <c r="J85" s="7" t="inlineStr"/>
     </row>
     <row r="86" ht="48" customHeight="1">
       <c r="A86" s="7" t="n">
@@ -4420,22 +4510,22 @@
       </c>
       <c r="B86" s="6" t="inlineStr">
         <is>
-          <t>11. Mở rộng giai đoạn 2-3</t>
+          <t>10. Hộp thư khách hàng</t>
         </is>
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>Tô màu chênh lệch giá so với catalog</t>
+          <t>Tổng hợp tin nhắn khách 19 cửa hàng vào một chỗ</t>
         </is>
       </c>
       <c r="D86" s="6" t="inlineStr">
         <is>
-          <t>Đỏ = thấp hơn catalog; vàng = bằng; tím = cao hơn.</t>
+          <t>Hệ thống tự kéo lời nhắn của khách (buyer message) khi khách đặt hàng và hiển thị: (a) trên trang đơn; (b) trên trang 'Hộp thư khách hàng' để Marketing/BA tìm xuyên cửa hàng.</t>
         </is>
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
-          <t>Kiểm soát giá</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="F86" s="7" t="inlineStr">
@@ -4453,7 +4543,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I86" s="6" t="inlineStr"/>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: chưa có dashboard tổng hợp tin nhắn khách trong ngày</t>
+        </is>
+      </c>
+      <c r="J86" s="7" t="inlineStr"/>
     </row>
     <row r="87" ht="48" customHeight="1">
       <c r="A87" s="7" t="n">
@@ -4466,12 +4561,12 @@
       </c>
       <c r="C87" s="6" t="inlineStr">
         <is>
-          <t>Cảnh báo đơn lệch giá tự động hằng ngày</t>
+          <t>Bảng kiểm soát giá (Pricing Audit) 25 cột</t>
         </is>
       </c>
       <c r="D87" s="6" t="inlineStr">
         <is>
-          <t>Mỗi sáng hệ thống lọc đơn vượt ngưỡng, gửi ping cho RD và tô màu trên dashboard.</t>
+          <t>RD nhập tay 6 cột (A-F), 19 cột còn lại tự lấy từ đơn. Hỗ trợ đa tiền tệ.</t>
         </is>
       </c>
       <c r="E87" s="6" t="inlineStr">
@@ -4495,6 +4590,7 @@
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr"/>
+      <c r="J87" s="7" t="inlineStr"/>
     </row>
     <row r="88" ht="48" customHeight="1">
       <c r="A88" s="7" t="n">
@@ -4507,27 +4603,27 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Catalog Dashboard riêng cho từng sản phẩm</t>
+          <t>Quy đổi giá đơn về EUR theo ngày đặt</t>
         </is>
       </c>
       <c r="D88" s="6" t="inlineStr">
         <is>
-          <t>Trên trang sản phẩm có template thiết kế, mockup, lịch sử bán.</t>
+          <t>Tự quy đổi USD/VND/CAD về EUR theo tỷ giá ngày đặt. Hiện 'Tổng tiền (EUR)'.</t>
         </is>
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Kiểm soát giá</t>
         </is>
       </c>
       <c r="F88" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G88" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 3</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H88" s="7" t="inlineStr">
@@ -4536,6 +4632,7 @@
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr"/>
+      <c r="J88" s="7" t="inlineStr"/>
     </row>
     <row r="89" ht="48" customHeight="1">
       <c r="A89" s="7" t="n">
@@ -4548,27 +4645,27 @@
       </c>
       <c r="C89" s="6" t="inlineStr">
         <is>
-          <t>Lưu template + mockup ngay trên sản phẩm</t>
+          <t>Tô màu chênh lệch giá so với catalog</t>
         </is>
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>Hai trường file trên sản phẩm: template gốc và mockup.</t>
+          <t>Đỏ = thấp hơn catalog; vàng = bằng; tím = cao hơn.</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>BA</t>
+          <t>Kiểm soát giá</t>
         </is>
       </c>
       <c r="F89" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 3</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H89" s="7" t="inlineStr">
@@ -4577,6 +4674,7 @@
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr"/>
+      <c r="J89" s="7" t="inlineStr"/>
     </row>
     <row r="90" ht="48" customHeight="1">
       <c r="A90" s="7" t="n">
@@ -4589,27 +4687,27 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>Trang scan barcode đơn giản cho PD</t>
+          <t>Cảnh báo đơn lệch giá tự động hằng ngày</t>
         </is>
       </c>
       <c r="D90" s="6" t="inlineStr">
         <is>
-          <t>Trang scan tối giản: ô input tự focus, enter là xác nhận.</t>
+          <t>Mỗi sáng hệ thống lọc đơn vượt ngưỡng, gửi ping cho RD và tô màu trên dashboard.</t>
         </is>
       </c>
       <c r="E90" s="6" t="inlineStr">
         <is>
-          <t>BA, Sản xuất</t>
+          <t>Kiểm soát giá</t>
         </is>
       </c>
       <c r="F90" s="7" t="inlineStr">
         <is>
-          <t>Thấp</t>
+          <t>Trung bình</t>
         </is>
       </c>
       <c r="G90" s="7" t="inlineStr">
         <is>
-          <t>Giai đoạn 3</t>
+          <t>Giai đoạn 2</t>
         </is>
       </c>
       <c r="H90" s="7" t="inlineStr">
@@ -4618,6 +4716,7 @@
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr"/>
+      <c r="J90" s="7" t="inlineStr"/>
     </row>
     <row r="91" ht="48" customHeight="1">
       <c r="A91" s="7" t="n">
@@ -4630,17 +4729,17 @@
       </c>
       <c r="C91" s="6" t="inlineStr">
         <is>
-          <t>Scan đồng bộ tất cả dashboard</t>
+          <t>Catalog Dashboard riêng cho từng sản phẩm</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Khi PD scan, mọi dashboard liên quan cập nhật trong vòng 5 giây.</t>
+          <t>Trên trang sản phẩm có template thiết kế, mockup, lịch sử bán.</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>BA, Sản xuất</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F91" s="7" t="inlineStr">
@@ -4659,6 +4758,7 @@
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr"/>
+      <c r="J91" s="7" t="inlineStr"/>
     </row>
     <row r="92" ht="48" customHeight="1">
       <c r="A92" s="7" t="n">
@@ -4671,17 +4771,17 @@
       </c>
       <c r="C92" s="6" t="inlineStr">
         <is>
-          <t>Tích hợp Amazon — đơn vào dashboard chung</t>
+          <t>Lưu template + mockup ngay trên sản phẩm</t>
         </is>
       </c>
       <c r="D92" s="6" t="inlineStr">
         <is>
-          <t>Kết nối Amazon Seller Central; đơn Amazon hiển thị chung Bảng Đơn hàng.</t>
+          <t>Hai trường file trên sản phẩm: template gốc và mockup.</t>
         </is>
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>BA</t>
         </is>
       </c>
       <c r="F92" s="7" t="inlineStr">
@@ -4700,6 +4800,7 @@
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr"/>
+      <c r="J92" s="7" t="inlineStr"/>
     </row>
     <row r="93" ht="48" customHeight="1">
       <c r="A93" s="7" t="n">
@@ -4712,17 +4813,17 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Mở Website Odoo và đưa đơn về dashboard chung</t>
+          <t>Trang scan barcode đơn giản cho PD</t>
         </is>
       </c>
       <c r="D93" s="6" t="inlineStr">
         <is>
-          <t>Bật module Website của Odoo; đơn website hiển thị chung Bảng Đơn hàng.</t>
+          <t>Trang scan tối giản: ô input tự focus, enter là xác nhận.</t>
         </is>
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
-          <t>Chủ dự án</t>
+          <t>BA, Sản xuất</t>
         </is>
       </c>
       <c r="F93" s="7" t="inlineStr">
@@ -4741,6 +4842,7 @@
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr"/>
+      <c r="J93" s="7" t="inlineStr"/>
     </row>
     <row r="94" ht="48" customHeight="1">
       <c r="A94" s="7" t="n">
@@ -4753,17 +4855,17 @@
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Hỗ trợ AI tổng hợp / trực quan hoá dữ liệu</t>
+          <t>Scan đồng bộ tất cả dashboard</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr">
         <is>
-          <t>Giai đoạn 1 chốt cấu trúc dữ liệu để các công cụ BI/AI đọc. Giai đoạn 3 mới triển khai phân tích, dự báo và trực quan hoá.</t>
+          <t>Khi PD scan, mọi dashboard liên quan cập nhật trong vòng 5 giây.</t>
         </is>
       </c>
       <c r="E94" s="6" t="inlineStr">
         <is>
-          <t>Marketing, BA, Sản xuất</t>
+          <t>BA, Sản xuất</t>
         </is>
       </c>
       <c r="F94" s="7" t="inlineStr">
@@ -4781,11 +4883,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I94" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: cần AI hỗ trợ trích xuất, tổng kết, trực quan hoá dữ liệu</t>
-        </is>
-      </c>
+      <c r="I94" s="6" t="inlineStr"/>
+      <c r="J94" s="7" t="inlineStr"/>
     </row>
     <row r="95" ht="48" customHeight="1">
       <c r="A95" s="7" t="n">
@@ -4793,17 +4892,17 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>12. Tồn kho nguyên liệu</t>
+          <t>11. Mở rộng giai đoạn 2-3</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Upload tồn kho nguyên liệu từ Excel</t>
+          <t>Tích hợp Amazon — đơn vào dashboard chung</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr">
         <is>
-          <t>PD upload Excel; hệ thống tạo tồn kho đầu kỳ.</t>
+          <t>Kết nối Amazon Seller Central; đơn Amazon hiển thị chung Bảng Đơn hàng.</t>
         </is>
       </c>
       <c r="E95" s="6" t="inlineStr">
@@ -4813,7 +4912,7 @@
       </c>
       <c r="F95" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G95" s="7" t="inlineStr">
@@ -4826,11 +4925,8 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I95" s="6" t="inlineStr">
-        <is>
-          <t>Tiếp thu phản hồi: nguyên liệu cập nhật hằng tháng</t>
-        </is>
-      </c>
+      <c r="I95" s="6" t="inlineStr"/>
+      <c r="J95" s="7" t="inlineStr"/>
     </row>
     <row r="96" ht="48" customHeight="1">
       <c r="A96" s="7" t="n">
@@ -4838,27 +4934,27 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>12. Tồn kho nguyên liệu</t>
+          <t>11. Mở rộng giai đoạn 2-3</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Tự trừ nguyên liệu khi đơn đến giai đoạn cuối</t>
+          <t>Mở Website Odoo và đưa đơn về dashboard chung</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr">
         <is>
-          <t>Khi đơn nhảy đến giai đoạn được đánh dấu 'Trừ kho', hệ thống tự trừ nguyên liệu theo định mức.</t>
+          <t>Bật module Website của Odoo; đơn website hiển thị chung Bảng Đơn hàng.</t>
         </is>
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>Chủ dự án</t>
         </is>
       </c>
       <c r="F96" s="7" t="inlineStr">
         <is>
-          <t>Trung bình</t>
+          <t>Thấp</t>
         </is>
       </c>
       <c r="G96" s="7" t="inlineStr">
@@ -4872,6 +4968,7 @@
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr"/>
+      <c r="J96" s="7" t="inlineStr"/>
     </row>
     <row r="97" ht="48" customHeight="1">
       <c r="A97" s="7" t="n">
@@ -4879,22 +4976,22 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>12. Tồn kho nguyên liệu</t>
+          <t>11. Mở rộng giai đoạn 2-3</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Dự báo tồn kho 1 / 3 / 12 tháng</t>
+          <t>Hỗ trợ AI tổng hợp / trực quan hoá dữ liệu</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr">
         <is>
-          <t>Bảng dự báo: tồn kho hiện tại đủ dùng bao lâu.</t>
+          <t>Giai đoạn 1 chốt cấu trúc dữ liệu để các công cụ BI/AI đọc. Giai đoạn 3 mới triển khai phân tích, dự báo và trực quan hoá.</t>
         </is>
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>Sản xuất</t>
+          <t>Marketing, BA, Sản xuất</t>
         </is>
       </c>
       <c r="F97" s="7" t="inlineStr">
@@ -4912,7 +5009,12 @@
           <t>Chưa bắt đầu</t>
         </is>
       </c>
-      <c r="I97" s="6" t="inlineStr"/>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: cần AI hỗ trợ trích xuất, tổng kết, trực quan hoá dữ liệu</t>
+        </is>
+      </c>
+      <c r="J97" s="7" t="inlineStr"/>
     </row>
     <row r="98" ht="48" customHeight="1">
       <c r="A98" s="7" t="n">
@@ -4925,39 +5027,170 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
+          <t>Upload tồn kho nguyên liệu từ Excel</t>
+        </is>
+      </c>
+      <c r="D98" s="6" t="inlineStr">
+        <is>
+          <t>PD upload Excel; hệ thống tạo tồn kho đầu kỳ.</t>
+        </is>
+      </c>
+      <c r="E98" s="6" t="inlineStr">
+        <is>
+          <t>Sản xuất</t>
+        </is>
+      </c>
+      <c r="F98" s="7" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G98" s="7" t="inlineStr">
+        <is>
+          <t>Giai đoạn 3</t>
+        </is>
+      </c>
+      <c r="H98" s="7" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="I98" s="6" t="inlineStr">
+        <is>
+          <t>Tiếp thu phản hồi: nguyên liệu cập nhật hằng tháng</t>
+        </is>
+      </c>
+      <c r="J98" s="7" t="inlineStr"/>
+    </row>
+    <row r="99" ht="48" customHeight="1">
+      <c r="A99" s="7" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>12. Tồn kho nguyên liệu</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>Tự trừ nguyên liệu khi đơn đến giai đoạn cuối</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>Khi đơn nhảy đến giai đoạn được đánh dấu 'Trừ kho', hệ thống tự trừ nguyên liệu theo định mức.</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="inlineStr">
+        <is>
+          <t>Sản xuất</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr">
+        <is>
+          <t>Trung bình</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="inlineStr">
+        <is>
+          <t>Giai đoạn 3</t>
+        </is>
+      </c>
+      <c r="H99" s="7" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr"/>
+      <c r="J99" s="7" t="inlineStr"/>
+    </row>
+    <row r="100" ht="48" customHeight="1">
+      <c r="A100" s="7" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>12. Tồn kho nguyên liệu</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Dự báo tồn kho 1 / 3 / 12 tháng</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr">
+        <is>
+          <t>Bảng dự báo: tồn kho hiện tại đủ dùng bao lâu.</t>
+        </is>
+      </c>
+      <c r="E100" s="6" t="inlineStr">
+        <is>
+          <t>Sản xuất</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>Thấp</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>Giai đoạn 3</t>
+        </is>
+      </c>
+      <c r="H100" s="7" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr"/>
+      <c r="J100" s="7" t="inlineStr"/>
+    </row>
+    <row r="101" ht="48" customHeight="1">
+      <c r="A101" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>12. Tồn kho nguyên liệu</t>
+        </is>
+      </c>
+      <c r="C101" s="6" t="inlineStr">
+        <is>
           <t>Cảnh báo nguyên liệu còn dưới 2 tháng</t>
         </is>
       </c>
-      <c r="D98" s="6" t="inlineStr">
+      <c r="D101" s="6" t="inlineStr">
         <is>
           <t>PD Lead nhận thông báo và dashboard tô đỏ những NVL sắp hết.</t>
         </is>
       </c>
-      <c r="E98" s="6" t="inlineStr">
+      <c r="E101" s="6" t="inlineStr">
         <is>
           <t>Sản xuất</t>
         </is>
       </c>
-      <c r="F98" s="7" t="inlineStr">
+      <c r="F101" s="7" t="inlineStr">
         <is>
           <t>Thấp</t>
         </is>
       </c>
-      <c r="G98" s="7" t="inlineStr">
+      <c r="G101" s="7" t="inlineStr">
         <is>
           <t>Giai đoạn 3</t>
         </is>
       </c>
-      <c r="H98" s="7" t="inlineStr">
-        <is>
-          <t>Chưa bắt đầu</t>
-        </is>
-      </c>
-      <c r="I98" s="6" t="inlineStr"/>
+      <c r="H101" s="7" t="inlineStr">
+        <is>
+          <t>Chưa bắt đầu</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr"/>
+      <c r="J101" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I98"/>
-  <conditionalFormatting sqref="F2:F98">
+  <autoFilter ref="A1:J101"/>
+  <conditionalFormatting sqref="F2:F101">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Cao"</formula>
     </cfRule>
@@ -4968,7 +5201,7 @@
       <formula>"Thấp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H98">
+  <conditionalFormatting sqref="H2:H101">
     <cfRule type="cellIs" priority="4" operator="equal" dxfId="2">
       <formula>"Hoàn thành"</formula>
     </cfRule>
@@ -4977,13 +5210,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="F2:F98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Cao,Trung bình,Thấp"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Giai đoạn 1,Giai đoạn 2,Giai đoạn 3"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="H2:H101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Chưa bắt đầu,Đang làm,Hoàn thành,Chặn"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
[mp006] docs: mark 58 owner items as Hoàn thành based on demo milestone
The 2026-05-08 first 12/12 GREEN drop-ship E2E run on demo confirms
58 items work end-to-end. Mark them Hoàn thành in xlsx so the owner
sees an honest progress snapshot.

- Add status_overrides.json sidecar (ten_ngan -> trạng thái)
- Wire build_catalog() to load it (defaults stay "Chưa bắt đầu")
- Tom_Tat dashboard COUNTIF formulas pick up the change live
- 3 new items (parity check, line-level dashboard, label photos)
  remain "Chưa bắt đầu" — not part of the demo milestone yet
</commit_message>
<xml_diff>
--- a/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
+++ b/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
@@ -992,7 +992,7 @@
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
@@ -1458,7 +1458,7 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
@@ -1500,7 +1500,7 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
@@ -1542,7 +1542,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
@@ -1584,7 +1584,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
@@ -1752,7 +1752,7 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
@@ -1878,7 +1878,7 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
@@ -1920,7 +1920,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
@@ -2088,7 +2088,7 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
@@ -2172,7 +2172,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
@@ -2214,7 +2214,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
@@ -2256,7 +2256,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr"/>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
@@ -2340,7 +2340,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
@@ -2466,7 +2466,7 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
@@ -2508,7 +2508,7 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
@@ -2550,7 +2550,7 @@
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
@@ -2634,7 +2634,7 @@
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="H54" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="H55" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="H56" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="H57" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="H62" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="H64" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -3948,7 +3948,7 @@
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
@@ -3990,7 +3990,7 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4036,7 +4036,7 @@
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
@@ -4204,7 +4204,7 @@
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr"/>
@@ -4288,7 +4288,7 @@
       </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr"/>
@@ -4330,7 +4330,7 @@
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
@@ -4372,7 +4372,7 @@
       </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
@@ -4414,7 +4414,7 @@
       </c>
       <c r="H83" s="7" t="inlineStr">
         <is>
-          <t>Chưa bắt đầu</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
[mp006] docs: sync 100 owner items to JIRA (12 epics + 100 stories)
JIRA topology mirrors xlsx structure:
- 12 Epics (one per Nhóm hạng mục group): ESTY-7..ESTY-18
- 100 Stories (one per row, parent-linked to its group epic): ESTY-19..ESTY-118
- Status synced: 58 Hoàn thành -> JIRA Done, 42 Chưa bắt đầu -> JIRA To Do
- xlsx column J back-filled with all 100 story keys

New deliverables:
- jira_sync.py: idempotent sync helper (direct JIRA REST v3, sleep-throttled)
- epic_key_map.json: nhom -> epic key mapping (skips already-pushed on re-run)
- jira_keys.json: ten_ngan -> story key mapping (loaded by build_owner_docs)

Re-running jira_sync.py is safe: skips entries already in epic_key_map /
jira_keys / draft frontmatter.
</commit_message>
<xml_diff>
--- a/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
+++ b/specs/006-master-plan/deliverables/Theo_Doi_Du_An_VN.xlsx
@@ -996,7 +996,11 @@
         </is>
       </c>
       <c r="I2" s="6" t="inlineStr"/>
-      <c r="J2" s="7" t="inlineStr"/>
+      <c r="J2" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-19</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="7" t="n">
@@ -1038,7 +1042,11 @@
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="7" t="inlineStr"/>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-20</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="48" customHeight="1">
       <c r="A4" s="7" t="n">
@@ -1080,7 +1088,11 @@
         </is>
       </c>
       <c r="I4" s="6" t="inlineStr"/>
-      <c r="J4" s="7" t="inlineStr"/>
+      <c r="J4" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-21</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="7" t="n">
@@ -1122,7 +1134,11 @@
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="7" t="inlineStr"/>
+      <c r="J5" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-22</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="48" customHeight="1">
       <c r="A6" s="7" t="n">
@@ -1164,7 +1180,11 @@
         </is>
       </c>
       <c r="I6" s="6" t="inlineStr"/>
-      <c r="J6" s="7" t="inlineStr"/>
+      <c r="J6" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-23</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="48" customHeight="1">
       <c r="A7" s="7" t="n">
@@ -1206,7 +1226,11 @@
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="7" t="inlineStr"/>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-24</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="7" t="n">
@@ -1248,7 +1272,11 @@
         </is>
       </c>
       <c r="I8" s="6" t="inlineStr"/>
-      <c r="J8" s="7" t="inlineStr"/>
+      <c r="J8" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-25</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="48" customHeight="1">
       <c r="A9" s="7" t="n">
@@ -1290,7 +1318,11 @@
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="7" t="inlineStr"/>
+      <c r="J9" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-26</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="48" customHeight="1">
       <c r="A10" s="7" t="n">
@@ -1336,7 +1368,11 @@
           <t>Đã đối chiếu thành công 12/12 đơn mẫu trên môi trường demo.</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr"/>
+      <c r="J10" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-27</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="7" t="n">
@@ -1378,7 +1414,11 @@
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="7" t="inlineStr"/>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-28</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -1420,7 +1460,11 @@
         </is>
       </c>
       <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr"/>
+      <c r="J12" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-29</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="48" customHeight="1">
       <c r="A13" s="7" t="n">
@@ -1462,7 +1506,11 @@
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="7" t="inlineStr"/>
+      <c r="J13" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-30</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="7" t="n">
@@ -1504,7 +1552,11 @@
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr"/>
-      <c r="J14" s="7" t="inlineStr"/>
+      <c r="J14" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-31</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="48" customHeight="1">
       <c r="A15" s="7" t="n">
@@ -1546,7 +1598,11 @@
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="7" t="inlineStr"/>
+      <c r="J15" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-32</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="7" t="n">
@@ -1588,7 +1644,11 @@
         </is>
       </c>
       <c r="I16" s="6" t="inlineStr"/>
-      <c r="J16" s="7" t="inlineStr"/>
+      <c r="J16" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-33</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="48" customHeight="1">
       <c r="A17" s="7" t="n">
@@ -1630,7 +1690,11 @@
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="7" t="inlineStr"/>
+      <c r="J17" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-34</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="48" customHeight="1">
       <c r="A18" s="7" t="n">
@@ -1672,7 +1736,11 @@
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="7" t="inlineStr"/>
+      <c r="J18" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-35</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="48" customHeight="1">
       <c r="A19" s="7" t="n">
@@ -1714,7 +1782,11 @@
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="7" t="inlineStr"/>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-36</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="48" customHeight="1">
       <c r="A20" s="7" t="n">
@@ -1756,7 +1828,11 @@
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="7" t="inlineStr"/>
+      <c r="J20" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-37</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="48" customHeight="1">
       <c r="A21" s="7" t="n">
@@ -1798,7 +1874,11 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="7" t="inlineStr"/>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-38</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="48" customHeight="1">
       <c r="A22" s="7" t="n">
@@ -1840,7 +1920,11 @@
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr"/>
-      <c r="J22" s="7" t="inlineStr"/>
+      <c r="J22" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-39</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="48" customHeight="1">
       <c r="A23" s="7" t="n">
@@ -1882,7 +1966,11 @@
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
-      <c r="J23" s="7" t="inlineStr"/>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-40</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="48" customHeight="1">
       <c r="A24" s="7" t="n">
@@ -1924,7 +2012,11 @@
         </is>
       </c>
       <c r="I24" s="6" t="inlineStr"/>
-      <c r="J24" s="7" t="inlineStr"/>
+      <c r="J24" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-41</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="48" customHeight="1">
       <c r="A25" s="7" t="n">
@@ -1966,7 +2058,11 @@
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="7" t="inlineStr"/>
+      <c r="J25" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-42</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="48" customHeight="1">
       <c r="A26" s="7" t="n">
@@ -2008,7 +2104,11 @@
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr"/>
-      <c r="J26" s="7" t="inlineStr"/>
+      <c r="J26" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-43</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="48" customHeight="1">
       <c r="A27" s="7" t="n">
@@ -2050,7 +2150,11 @@
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
-      <c r="J27" s="7" t="inlineStr"/>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-44</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="48" customHeight="1">
       <c r="A28" s="7" t="n">
@@ -2092,7 +2196,11 @@
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr"/>
-      <c r="J28" s="7" t="inlineStr"/>
+      <c r="J28" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-45</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="48" customHeight="1">
       <c r="A29" s="7" t="n">
@@ -2134,7 +2242,11 @@
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr"/>
-      <c r="J29" s="7" t="inlineStr"/>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-46</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="48" customHeight="1">
       <c r="A30" s="7" t="n">
@@ -2176,7 +2288,11 @@
         </is>
       </c>
       <c r="I30" s="6" t="inlineStr"/>
-      <c r="J30" s="7" t="inlineStr"/>
+      <c r="J30" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-47</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="A31" s="7" t="n">
@@ -2218,7 +2334,11 @@
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr"/>
-      <c r="J31" s="7" t="inlineStr"/>
+      <c r="J31" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-48</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="48" customHeight="1">
       <c r="A32" s="7" t="n">
@@ -2260,7 +2380,11 @@
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr"/>
-      <c r="J32" s="7" t="inlineStr"/>
+      <c r="J32" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-49</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="48" customHeight="1">
       <c r="A33" s="7" t="n">
@@ -2302,7 +2426,11 @@
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr"/>
-      <c r="J33" s="7" t="inlineStr"/>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-50</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="48" customHeight="1">
       <c r="A34" s="7" t="n">
@@ -2344,7 +2472,11 @@
         </is>
       </c>
       <c r="I34" s="6" t="inlineStr"/>
-      <c r="J34" s="7" t="inlineStr"/>
+      <c r="J34" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-51</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="48" customHeight="1">
       <c r="A35" s="7" t="n">
@@ -2386,7 +2518,11 @@
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr"/>
-      <c r="J35" s="7" t="inlineStr"/>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-52</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="48" customHeight="1">
       <c r="A36" s="7" t="n">
@@ -2428,7 +2564,11 @@
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr"/>
-      <c r="J36" s="7" t="inlineStr"/>
+      <c r="J36" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-53</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="48" customHeight="1">
       <c r="A37" s="7" t="n">
@@ -2470,7 +2610,11 @@
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr"/>
-      <c r="J37" s="7" t="inlineStr"/>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-54</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="48" customHeight="1">
       <c r="A38" s="7" t="n">
@@ -2512,7 +2656,11 @@
         </is>
       </c>
       <c r="I38" s="6" t="inlineStr"/>
-      <c r="J38" s="7" t="inlineStr"/>
+      <c r="J38" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-55</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="48" customHeight="1">
       <c r="A39" s="7" t="n">
@@ -2554,7 +2702,11 @@
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr"/>
-      <c r="J39" s="7" t="inlineStr"/>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-56</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="48" customHeight="1">
       <c r="A40" s="7" t="n">
@@ -2596,7 +2748,11 @@
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr"/>
-      <c r="J40" s="7" t="inlineStr"/>
+      <c r="J40" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-57</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="48" customHeight="1">
       <c r="A41" s="7" t="n">
@@ -2638,7 +2794,11 @@
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr"/>
-      <c r="J41" s="7" t="inlineStr"/>
+      <c r="J41" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-58</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="48" customHeight="1">
       <c r="A42" s="7" t="n">
@@ -2680,7 +2840,11 @@
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr"/>
-      <c r="J42" s="7" t="inlineStr"/>
+      <c r="J42" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-59</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="48" customHeight="1">
       <c r="A43" s="7" t="n">
@@ -2722,7 +2886,11 @@
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr"/>
-      <c r="J43" s="7" t="inlineStr"/>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-60</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="48" customHeight="1">
       <c r="A44" s="7" t="n">
@@ -2764,7 +2932,11 @@
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr"/>
-      <c r="J44" s="7" t="inlineStr"/>
+      <c r="J44" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-61</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="48" customHeight="1">
       <c r="A45" s="7" t="n">
@@ -2806,7 +2978,11 @@
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr"/>
-      <c r="J45" s="7" t="inlineStr"/>
+      <c r="J45" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-62</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="48" customHeight="1">
       <c r="A46" s="7" t="n">
@@ -2848,7 +3024,11 @@
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr"/>
-      <c r="J46" s="7" t="inlineStr"/>
+      <c r="J46" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-63</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="48" customHeight="1">
       <c r="A47" s="7" t="n">
@@ -2894,7 +3074,11 @@
           <t>Tiếp thu phản hồi của Owner</t>
         </is>
       </c>
-      <c r="J47" s="7" t="inlineStr"/>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-64</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="48" customHeight="1">
       <c r="A48" s="7" t="n">
@@ -2936,7 +3120,11 @@
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr"/>
-      <c r="J48" s="7" t="inlineStr"/>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-65</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="48" customHeight="1">
       <c r="A49" s="7" t="n">
@@ -2978,7 +3166,11 @@
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr"/>
-      <c r="J49" s="7" t="inlineStr"/>
+      <c r="J49" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-66</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="48" customHeight="1">
       <c r="A50" s="7" t="n">
@@ -3020,7 +3212,11 @@
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr"/>
-      <c r="J50" s="7" t="inlineStr"/>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-67</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="48" customHeight="1">
       <c r="A51" s="7" t="n">
@@ -3062,7 +3258,11 @@
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr"/>
-      <c r="J51" s="7" t="inlineStr"/>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-68</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="48" customHeight="1">
       <c r="A52" s="7" t="n">
@@ -3104,7 +3304,11 @@
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr"/>
-      <c r="J52" s="7" t="inlineStr"/>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-69</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="48" customHeight="1">
       <c r="A53" s="7" t="n">
@@ -3146,7 +3350,11 @@
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr"/>
-      <c r="J53" s="7" t="inlineStr"/>
+      <c r="J53" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-70</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="48" customHeight="1">
       <c r="A54" s="7" t="n">
@@ -3188,7 +3396,11 @@
         </is>
       </c>
       <c r="I54" s="6" t="inlineStr"/>
-      <c r="J54" s="7" t="inlineStr"/>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-71</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="48" customHeight="1">
       <c r="A55" s="7" t="n">
@@ -3230,7 +3442,11 @@
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr"/>
-      <c r="J55" s="7" t="inlineStr"/>
+      <c r="J55" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-72</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="48" customHeight="1">
       <c r="A56" s="7" t="n">
@@ -3272,7 +3488,11 @@
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr"/>
-      <c r="J56" s="7" t="inlineStr"/>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-73</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="48" customHeight="1">
       <c r="A57" s="7" t="n">
@@ -3314,7 +3534,11 @@
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr"/>
-      <c r="J57" s="7" t="inlineStr"/>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-74</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="48" customHeight="1">
       <c r="A58" s="7" t="n">
@@ -3356,7 +3580,11 @@
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr"/>
-      <c r="J58" s="7" t="inlineStr"/>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-75</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="48" customHeight="1">
       <c r="A59" s="7" t="n">
@@ -3398,7 +3626,11 @@
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr"/>
-      <c r="J59" s="7" t="inlineStr"/>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-76</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="48" customHeight="1">
       <c r="A60" s="7" t="n">
@@ -3440,7 +3672,11 @@
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr"/>
-      <c r="J60" s="7" t="inlineStr"/>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-77</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="48" customHeight="1">
       <c r="A61" s="7" t="n">
@@ -3482,7 +3718,11 @@
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr"/>
-      <c r="J61" s="7" t="inlineStr"/>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-78</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="48" customHeight="1">
       <c r="A62" s="7" t="n">
@@ -3528,7 +3768,11 @@
           <t>Tiếp thu phản hồi: thay vì copy tay từ file logistics sang Google Excel</t>
         </is>
       </c>
-      <c r="J62" s="7" t="inlineStr"/>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-79</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="48" customHeight="1">
       <c r="A63" s="7" t="n">
@@ -3570,7 +3814,11 @@
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr"/>
-      <c r="J63" s="7" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-80</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="48" customHeight="1">
       <c r="A64" s="7" t="n">
@@ -3612,7 +3860,11 @@
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr"/>
-      <c r="J64" s="7" t="inlineStr"/>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-81</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="48" customHeight="1">
       <c r="A65" s="7" t="n">
@@ -3654,7 +3906,11 @@
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr"/>
-      <c r="J65" s="7" t="inlineStr"/>
+      <c r="J65" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-82</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="48" customHeight="1">
       <c r="A66" s="7" t="n">
@@ -3696,7 +3952,11 @@
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr"/>
-      <c r="J66" s="7" t="inlineStr"/>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-83</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="48" customHeight="1">
       <c r="A67" s="7" t="n">
@@ -3738,7 +3998,11 @@
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr"/>
-      <c r="J67" s="7" t="inlineStr"/>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-84</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="48" customHeight="1">
       <c r="A68" s="7" t="n">
@@ -3780,7 +4044,11 @@
         </is>
       </c>
       <c r="I68" s="6" t="inlineStr"/>
-      <c r="J68" s="7" t="inlineStr"/>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-85</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="48" customHeight="1">
       <c r="A69" s="7" t="n">
@@ -3822,7 +4090,11 @@
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr"/>
-      <c r="J69" s="7" t="inlineStr"/>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-86</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="48" customHeight="1">
       <c r="A70" s="7" t="n">
@@ -3864,7 +4136,11 @@
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr"/>
-      <c r="J70" s="7" t="inlineStr"/>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-87</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="48" customHeight="1">
       <c r="A71" s="7" t="n">
@@ -3910,7 +4186,11 @@
           <t>Tiếp thu phản hồi: file 8MB không gửi được Discord, hay bị thất lạc, mất thời gian tải lên-tải xuống nhiều lần</t>
         </is>
       </c>
-      <c r="J71" s="7" t="inlineStr"/>
+      <c r="J71" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-88</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="48" customHeight="1">
       <c r="A72" s="7" t="n">
@@ -3952,7 +4232,11 @@
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr"/>
-      <c r="J72" s="7" t="inlineStr"/>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-89</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="48" customHeight="1">
       <c r="A73" s="7" t="n">
@@ -3998,7 +4282,11 @@
           <t>Tiếp thu phản hồi: PD mất nhiều thời gian search mã đơn, download file, sắp lên Photoshop</t>
         </is>
       </c>
-      <c r="J73" s="7" t="inlineStr"/>
+      <c r="J73" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-90</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="48" customHeight="1">
       <c r="A74" s="7" t="n">
@@ -4040,7 +4328,11 @@
         </is>
       </c>
       <c r="I74" s="6" t="inlineStr"/>
-      <c r="J74" s="7" t="inlineStr"/>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-91</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="48" customHeight="1">
       <c r="A75" s="7" t="n">
@@ -4082,7 +4374,11 @@
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr"/>
-      <c r="J75" s="7" t="inlineStr"/>
+      <c r="J75" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-92</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="48" customHeight="1">
       <c r="A76" s="7" t="n">
@@ -4124,7 +4420,11 @@
         </is>
       </c>
       <c r="I76" s="6" t="inlineStr"/>
-      <c r="J76" s="7" t="inlineStr"/>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-93</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="48" customHeight="1">
       <c r="A77" s="7" t="n">
@@ -4166,7 +4466,11 @@
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr"/>
-      <c r="J77" s="7" t="inlineStr"/>
+      <c r="J77" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-94</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="48" customHeight="1">
       <c r="A78" s="7" t="n">
@@ -4208,7 +4512,11 @@
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr"/>
-      <c r="J78" s="7" t="inlineStr"/>
+      <c r="J78" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-95</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="48" customHeight="1">
       <c r="A79" s="7" t="n">
@@ -4250,7 +4558,11 @@
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr"/>
-      <c r="J79" s="7" t="inlineStr"/>
+      <c r="J79" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-96</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="48" customHeight="1">
       <c r="A80" s="7" t="n">
@@ -4292,7 +4604,11 @@
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr"/>
-      <c r="J80" s="7" t="inlineStr"/>
+      <c r="J80" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-97</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="48" customHeight="1">
       <c r="A81" s="7" t="n">
@@ -4334,7 +4650,11 @@
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr"/>
-      <c r="J81" s="7" t="inlineStr"/>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-98</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="48" customHeight="1">
       <c r="A82" s="7" t="n">
@@ -4376,7 +4696,11 @@
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr"/>
-      <c r="J82" s="7" t="inlineStr"/>
+      <c r="J82" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-99</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="48" customHeight="1">
       <c r="A83" s="7" t="n">
@@ -4418,7 +4742,11 @@
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr"/>
-      <c r="J83" s="7" t="inlineStr"/>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-100</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="48" customHeight="1">
       <c r="A84" s="7" t="n">
@@ -4460,7 +4788,11 @@
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr"/>
-      <c r="J84" s="7" t="inlineStr"/>
+      <c r="J84" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-101</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="48" customHeight="1">
       <c r="A85" s="7" t="n">
@@ -4502,7 +4834,11 @@
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr"/>
-      <c r="J85" s="7" t="inlineStr"/>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-102</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="48" customHeight="1">
       <c r="A86" s="7" t="n">
@@ -4548,7 +4884,11 @@
           <t>Tiếp thu phản hồi: chưa có dashboard tổng hợp tin nhắn khách trong ngày</t>
         </is>
       </c>
-      <c r="J86" s="7" t="inlineStr"/>
+      <c r="J86" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-103</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="48" customHeight="1">
       <c r="A87" s="7" t="n">
@@ -4590,7 +4930,11 @@
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr"/>
-      <c r="J87" s="7" t="inlineStr"/>
+      <c r="J87" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-104</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="48" customHeight="1">
       <c r="A88" s="7" t="n">
@@ -4632,7 +4976,11 @@
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr"/>
-      <c r="J88" s="7" t="inlineStr"/>
+      <c r="J88" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-105</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="48" customHeight="1">
       <c r="A89" s="7" t="n">
@@ -4674,7 +5022,11 @@
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr"/>
-      <c r="J89" s="7" t="inlineStr"/>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-106</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="48" customHeight="1">
       <c r="A90" s="7" t="n">
@@ -4716,7 +5068,11 @@
         </is>
       </c>
       <c r="I90" s="6" t="inlineStr"/>
-      <c r="J90" s="7" t="inlineStr"/>
+      <c r="J90" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-107</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="48" customHeight="1">
       <c r="A91" s="7" t="n">
@@ -4758,7 +5114,11 @@
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr"/>
-      <c r="J91" s="7" t="inlineStr"/>
+      <c r="J91" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-108</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="48" customHeight="1">
       <c r="A92" s="7" t="n">
@@ -4800,7 +5160,11 @@
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr"/>
-      <c r="J92" s="7" t="inlineStr"/>
+      <c r="J92" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-109</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="48" customHeight="1">
       <c r="A93" s="7" t="n">
@@ -4842,7 +5206,11 @@
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr"/>
-      <c r="J93" s="7" t="inlineStr"/>
+      <c r="J93" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-110</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="48" customHeight="1">
       <c r="A94" s="7" t="n">
@@ -4884,7 +5252,11 @@
         </is>
       </c>
       <c r="I94" s="6" t="inlineStr"/>
-      <c r="J94" s="7" t="inlineStr"/>
+      <c r="J94" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-111</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="48" customHeight="1">
       <c r="A95" s="7" t="n">
@@ -4926,7 +5298,11 @@
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr"/>
-      <c r="J95" s="7" t="inlineStr"/>
+      <c r="J95" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-112</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="48" customHeight="1">
       <c r="A96" s="7" t="n">
@@ -4968,7 +5344,11 @@
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr"/>
-      <c r="J96" s="7" t="inlineStr"/>
+      <c r="J96" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-113</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="48" customHeight="1">
       <c r="A97" s="7" t="n">
@@ -5014,7 +5394,11 @@
           <t>Tiếp thu phản hồi: cần AI hỗ trợ trích xuất, tổng kết, trực quan hoá dữ liệu</t>
         </is>
       </c>
-      <c r="J97" s="7" t="inlineStr"/>
+      <c r="J97" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-114</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="48" customHeight="1">
       <c r="A98" s="7" t="n">
@@ -5060,7 +5444,11 @@
           <t>Tiếp thu phản hồi: nguyên liệu cập nhật hằng tháng</t>
         </is>
       </c>
-      <c r="J98" s="7" t="inlineStr"/>
+      <c r="J98" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-115</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="48" customHeight="1">
       <c r="A99" s="7" t="n">
@@ -5102,7 +5490,11 @@
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr"/>
-      <c r="J99" s="7" t="inlineStr"/>
+      <c r="J99" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-116</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="48" customHeight="1">
       <c r="A100" s="7" t="n">
@@ -5144,7 +5536,11 @@
         </is>
       </c>
       <c r="I100" s="6" t="inlineStr"/>
-      <c r="J100" s="7" t="inlineStr"/>
+      <c r="J100" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-117</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="48" customHeight="1">
       <c r="A101" s="7" t="n">
@@ -5186,7 +5582,11 @@
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr"/>
-      <c r="J101" s="7" t="inlineStr"/>
+      <c r="J101" s="7" t="inlineStr">
+        <is>
+          <t>ESTY-118</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J101"/>

</xml_diff>